<commit_message>
Clear dummy cost values from yellow input cells
Removed hardcoded default cost figures (人件費/燃料費/車両維持費/中間処理費等)
from 案件別採算 sheet. Cells are now blank to clearly indicate where actual
data still needs to be entered.

https://claude.ai/code/session_01BgHAFjDQSmbvXBnKUF79fq
</commit_message>
<xml_diff>
--- a/sacure_採算管理_v4_ルート別案件別.xlsx
+++ b/sacure_採算管理_v4_ルート別案件別.xlsx
@@ -1082,27 +1082,13 @@
         <f>D5+E5+F5+G5</f>
         <v/>
       </c>
-      <c r="I5" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O5" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I5" s="12" t="n"/>
+      <c r="J5" s="12" t="n"/>
+      <c r="K5" s="12" t="n"/>
+      <c r="L5" s="12" t="n"/>
+      <c r="M5" s="12" t="n"/>
+      <c r="N5" s="12" t="n"/>
+      <c r="O5" s="12" t="n"/>
       <c r="P5" s="13">
         <f>I5+J5+K5+L5+M5+N5+O5</f>
         <v/>
@@ -1161,27 +1147,13 @@
         <f>D6+E6+F6+G6</f>
         <v/>
       </c>
-      <c r="I6" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O6" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I6" s="12" t="n"/>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="12" t="n"/>
+      <c r="L6" s="12" t="n"/>
+      <c r="M6" s="12" t="n"/>
+      <c r="N6" s="12" t="n"/>
+      <c r="O6" s="12" t="n"/>
       <c r="P6" s="13">
         <f>I6+J6+K6+L6+M6+N6+O6</f>
         <v/>
@@ -1239,27 +1211,13 @@
         <f>D7+E7+F7+G7</f>
         <v/>
       </c>
-      <c r="I7" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J7" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K7" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L7" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M7" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N7" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O7" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="12" t="n"/>
+      <c r="L7" s="12" t="n"/>
+      <c r="M7" s="12" t="n"/>
+      <c r="N7" s="12" t="n"/>
+      <c r="O7" s="12" t="n"/>
       <c r="P7" s="13">
         <f>I7+J7+K7+L7+M7+N7+O7</f>
         <v/>
@@ -1317,27 +1275,13 @@
         <f>D8+E8+F8+G8</f>
         <v/>
       </c>
-      <c r="I8" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J8" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K8" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L8" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M8" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N8" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O8" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="12" t="n"/>
+      <c r="L8" s="12" t="n"/>
+      <c r="M8" s="12" t="n"/>
+      <c r="N8" s="12" t="n"/>
+      <c r="O8" s="12" t="n"/>
       <c r="P8" s="13">
         <f>I8+J8+K8+L8+M8+N8+O8</f>
         <v/>
@@ -1395,27 +1339,13 @@
         <f>D9+E9+F9+G9</f>
         <v/>
       </c>
-      <c r="I9" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O9" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="12" t="n"/>
+      <c r="L9" s="12" t="n"/>
+      <c r="M9" s="12" t="n"/>
+      <c r="N9" s="12" t="n"/>
+      <c r="O9" s="12" t="n"/>
       <c r="P9" s="13">
         <f>I9+J9+K9+L9+M9+N9+O9</f>
         <v/>
@@ -1473,27 +1403,13 @@
         <f>D10+E10+F10+G10</f>
         <v/>
       </c>
-      <c r="I10" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M10" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N10" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O10" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="12" t="n"/>
+      <c r="L10" s="12" t="n"/>
+      <c r="M10" s="12" t="n"/>
+      <c r="N10" s="12" t="n"/>
+      <c r="O10" s="12" t="n"/>
       <c r="P10" s="13">
         <f>I10+J10+K10+L10+M10+N10+O10</f>
         <v/>
@@ -1551,27 +1467,13 @@
         <f>D11+E11+F11+G11</f>
         <v/>
       </c>
-      <c r="I11" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O11" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="12" t="n"/>
+      <c r="L11" s="12" t="n"/>
+      <c r="M11" s="12" t="n"/>
+      <c r="N11" s="12" t="n"/>
+      <c r="O11" s="12" t="n"/>
       <c r="P11" s="13">
         <f>I11+J11+K11+L11+M11+N11+O11</f>
         <v/>
@@ -1629,27 +1531,13 @@
         <f>D12+E12+F12+G12</f>
         <v/>
       </c>
-      <c r="I12" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O12" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="12" t="n"/>
+      <c r="L12" s="12" t="n"/>
+      <c r="M12" s="12" t="n"/>
+      <c r="N12" s="12" t="n"/>
+      <c r="O12" s="12" t="n"/>
       <c r="P12" s="13">
         <f>I12+J12+K12+L12+M12+N12+O12</f>
         <v/>
@@ -1707,27 +1595,13 @@
         <f>D13+E13+F13+G13</f>
         <v/>
       </c>
-      <c r="I13" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J13" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K13" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M13" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N13" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O13" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="12" t="n"/>
+      <c r="L13" s="12" t="n"/>
+      <c r="M13" s="12" t="n"/>
+      <c r="N13" s="12" t="n"/>
+      <c r="O13" s="12" t="n"/>
       <c r="P13" s="13">
         <f>I13+J13+K13+L13+M13+N13+O13</f>
         <v/>
@@ -1785,27 +1659,13 @@
         <f>D14+E14+F14+G14</f>
         <v/>
       </c>
-      <c r="I14" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J14" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K14" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M14" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N14" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O14" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I14" s="12" t="n"/>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="12" t="n"/>
+      <c r="L14" s="12" t="n"/>
+      <c r="M14" s="12" t="n"/>
+      <c r="N14" s="12" t="n"/>
+      <c r="O14" s="12" t="n"/>
       <c r="P14" s="13">
         <f>I14+J14+K14+L14+M14+N14+O14</f>
         <v/>
@@ -1863,27 +1723,13 @@
         <f>D15+E15+F15+G15</f>
         <v/>
       </c>
-      <c r="I15" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N15" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O15" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I15" s="12" t="n"/>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="12" t="n"/>
+      <c r="L15" s="12" t="n"/>
+      <c r="M15" s="12" t="n"/>
+      <c r="N15" s="12" t="n"/>
+      <c r="O15" s="12" t="n"/>
       <c r="P15" s="13">
         <f>I15+J15+K15+L15+M15+N15+O15</f>
         <v/>
@@ -1941,27 +1787,13 @@
         <f>D16+E16+F16+G16</f>
         <v/>
       </c>
-      <c r="I16" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M16" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N16" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O16" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I16" s="12" t="n"/>
+      <c r="J16" s="12" t="n"/>
+      <c r="K16" s="12" t="n"/>
+      <c r="L16" s="12" t="n"/>
+      <c r="M16" s="12" t="n"/>
+      <c r="N16" s="12" t="n"/>
+      <c r="O16" s="12" t="n"/>
       <c r="P16" s="13">
         <f>I16+J16+K16+L16+M16+N16+O16</f>
         <v/>
@@ -2019,27 +1851,13 @@
         <f>D17+E17+F17+G17</f>
         <v/>
       </c>
-      <c r="I17" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O17" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="12" t="n"/>
+      <c r="L17" s="12" t="n"/>
+      <c r="M17" s="12" t="n"/>
+      <c r="N17" s="12" t="n"/>
+      <c r="O17" s="12" t="n"/>
       <c r="P17" s="13">
         <f>I17+J17+K17+L17+M17+N17+O17</f>
         <v/>
@@ -2097,27 +1915,13 @@
         <f>D18+E18+F18+G18</f>
         <v/>
       </c>
-      <c r="I18" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O18" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I18" s="12" t="n"/>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="12" t="n"/>
+      <c r="L18" s="12" t="n"/>
+      <c r="M18" s="12" t="n"/>
+      <c r="N18" s="12" t="n"/>
+      <c r="O18" s="12" t="n"/>
       <c r="P18" s="13">
         <f>I18+J18+K18+L18+M18+N18+O18</f>
         <v/>
@@ -2175,27 +1979,13 @@
         <f>D19+E19+F19+G19</f>
         <v/>
       </c>
-      <c r="I19" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J19" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K19" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L19" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M19" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N19" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O19" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I19" s="12" t="n"/>
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="12" t="n"/>
+      <c r="L19" s="12" t="n"/>
+      <c r="M19" s="12" t="n"/>
+      <c r="N19" s="12" t="n"/>
+      <c r="O19" s="12" t="n"/>
       <c r="P19" s="13">
         <f>I19+J19+K19+L19+M19+N19+O19</f>
         <v/>
@@ -2253,27 +2043,13 @@
         <f>D20+E20+F20+G20</f>
         <v/>
       </c>
-      <c r="I20" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J20" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K20" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L20" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M20" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N20" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O20" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I20" s="12" t="n"/>
+      <c r="J20" s="12" t="n"/>
+      <c r="K20" s="12" t="n"/>
+      <c r="L20" s="12" t="n"/>
+      <c r="M20" s="12" t="n"/>
+      <c r="N20" s="12" t="n"/>
+      <c r="O20" s="12" t="n"/>
       <c r="P20" s="13">
         <f>I20+J20+K20+L20+M20+N20+O20</f>
         <v/>
@@ -2331,27 +2107,13 @@
         <f>D21+E21+F21+G21</f>
         <v/>
       </c>
-      <c r="I21" s="12" t="n">
-        <v>680000</v>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>185000</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>620000</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>45000</v>
-      </c>
-      <c r="O21" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="I21" s="12" t="n"/>
+      <c r="J21" s="12" t="n"/>
+      <c r="K21" s="12" t="n"/>
+      <c r="L21" s="12" t="n"/>
+      <c r="M21" s="12" t="n"/>
+      <c r="N21" s="12" t="n"/>
+      <c r="O21" s="12" t="n"/>
       <c r="P21" s="13">
         <f>I21+J21+K21+L21+M21+N21+O21</f>
         <v/>
@@ -2431,27 +2193,13 @@
         <f>D23+E23+F23+G23</f>
         <v/>
       </c>
-      <c r="I23" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M23" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N23" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O23" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I23" s="12" t="n"/>
+      <c r="J23" s="12" t="n"/>
+      <c r="K23" s="12" t="n"/>
+      <c r="L23" s="12" t="n"/>
+      <c r="M23" s="12" t="n"/>
+      <c r="N23" s="12" t="n"/>
+      <c r="O23" s="12" t="n"/>
       <c r="P23" s="13">
         <f>I23+J23+K23+L23+M23+N23+O23</f>
         <v/>
@@ -2510,27 +2258,13 @@
         <f>D24+E24+F24+G24</f>
         <v/>
       </c>
-      <c r="I24" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J24" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K24" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M24" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N24" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O24" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I24" s="12" t="n"/>
+      <c r="J24" s="12" t="n"/>
+      <c r="K24" s="12" t="n"/>
+      <c r="L24" s="12" t="n"/>
+      <c r="M24" s="12" t="n"/>
+      <c r="N24" s="12" t="n"/>
+      <c r="O24" s="12" t="n"/>
       <c r="P24" s="13">
         <f>I24+J24+K24+L24+M24+N24+O24</f>
         <v/>
@@ -2588,27 +2322,13 @@
         <f>D25+E25+F25+G25</f>
         <v/>
       </c>
-      <c r="I25" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J25" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K25" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L25" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M25" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N25" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O25" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I25" s="12" t="n"/>
+      <c r="J25" s="12" t="n"/>
+      <c r="K25" s="12" t="n"/>
+      <c r="L25" s="12" t="n"/>
+      <c r="M25" s="12" t="n"/>
+      <c r="N25" s="12" t="n"/>
+      <c r="O25" s="12" t="n"/>
       <c r="P25" s="13">
         <f>I25+J25+K25+L25+M25+N25+O25</f>
         <v/>
@@ -2666,27 +2386,13 @@
         <f>D26+E26+F26+G26</f>
         <v/>
       </c>
-      <c r="I26" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J26" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K26" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L26" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M26" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N26" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O26" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I26" s="12" t="n"/>
+      <c r="J26" s="12" t="n"/>
+      <c r="K26" s="12" t="n"/>
+      <c r="L26" s="12" t="n"/>
+      <c r="M26" s="12" t="n"/>
+      <c r="N26" s="12" t="n"/>
+      <c r="O26" s="12" t="n"/>
       <c r="P26" s="13">
         <f>I26+J26+K26+L26+M26+N26+O26</f>
         <v/>
@@ -2744,27 +2450,13 @@
         <f>D27+E27+F27+G27</f>
         <v/>
       </c>
-      <c r="I27" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J27" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K27" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L27" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M27" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O27" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I27" s="12" t="n"/>
+      <c r="J27" s="12" t="n"/>
+      <c r="K27" s="12" t="n"/>
+      <c r="L27" s="12" t="n"/>
+      <c r="M27" s="12" t="n"/>
+      <c r="N27" s="12" t="n"/>
+      <c r="O27" s="12" t="n"/>
       <c r="P27" s="13">
         <f>I27+J27+K27+L27+M27+N27+O27</f>
         <v/>
@@ -2822,27 +2514,13 @@
         <f>D28+E28+F28+G28</f>
         <v/>
       </c>
-      <c r="I28" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J28" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K28" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L28" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M28" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O28" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I28" s="12" t="n"/>
+      <c r="J28" s="12" t="n"/>
+      <c r="K28" s="12" t="n"/>
+      <c r="L28" s="12" t="n"/>
+      <c r="M28" s="12" t="n"/>
+      <c r="N28" s="12" t="n"/>
+      <c r="O28" s="12" t="n"/>
       <c r="P28" s="13">
         <f>I28+J28+K28+L28+M28+N28+O28</f>
         <v/>
@@ -2900,27 +2578,13 @@
         <f>D29+E29+F29+G29</f>
         <v/>
       </c>
-      <c r="I29" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J29" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K29" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L29" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M29" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N29" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O29" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I29" s="12" t="n"/>
+      <c r="J29" s="12" t="n"/>
+      <c r="K29" s="12" t="n"/>
+      <c r="L29" s="12" t="n"/>
+      <c r="M29" s="12" t="n"/>
+      <c r="N29" s="12" t="n"/>
+      <c r="O29" s="12" t="n"/>
       <c r="P29" s="13">
         <f>I29+J29+K29+L29+M29+N29+O29</f>
         <v/>
@@ -2978,27 +2642,13 @@
         <f>D30+E30+F30+G30</f>
         <v/>
       </c>
-      <c r="I30" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J30" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K30" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L30" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M30" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N30" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O30" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I30" s="12" t="n"/>
+      <c r="J30" s="12" t="n"/>
+      <c r="K30" s="12" t="n"/>
+      <c r="L30" s="12" t="n"/>
+      <c r="M30" s="12" t="n"/>
+      <c r="N30" s="12" t="n"/>
+      <c r="O30" s="12" t="n"/>
       <c r="P30" s="13">
         <f>I30+J30+K30+L30+M30+N30+O30</f>
         <v/>
@@ -3056,27 +2706,13 @@
         <f>D31+E31+F31+G31</f>
         <v/>
       </c>
-      <c r="I31" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J31" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K31" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L31" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M31" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N31" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O31" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I31" s="12" t="n"/>
+      <c r="J31" s="12" t="n"/>
+      <c r="K31" s="12" t="n"/>
+      <c r="L31" s="12" t="n"/>
+      <c r="M31" s="12" t="n"/>
+      <c r="N31" s="12" t="n"/>
+      <c r="O31" s="12" t="n"/>
       <c r="P31" s="13">
         <f>I31+J31+K31+L31+M31+N31+O31</f>
         <v/>
@@ -3134,27 +2770,13 @@
         <f>D32+E32+F32+G32</f>
         <v/>
       </c>
-      <c r="I32" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J32" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K32" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L32" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M32" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N32" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O32" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I32" s="12" t="n"/>
+      <c r="J32" s="12" t="n"/>
+      <c r="K32" s="12" t="n"/>
+      <c r="L32" s="12" t="n"/>
+      <c r="M32" s="12" t="n"/>
+      <c r="N32" s="12" t="n"/>
+      <c r="O32" s="12" t="n"/>
       <c r="P32" s="13">
         <f>I32+J32+K32+L32+M32+N32+O32</f>
         <v/>
@@ -3212,27 +2834,13 @@
         <f>D33+E33+F33+G33</f>
         <v/>
       </c>
-      <c r="I33" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J33" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K33" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L33" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M33" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N33" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O33" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I33" s="12" t="n"/>
+      <c r="J33" s="12" t="n"/>
+      <c r="K33" s="12" t="n"/>
+      <c r="L33" s="12" t="n"/>
+      <c r="M33" s="12" t="n"/>
+      <c r="N33" s="12" t="n"/>
+      <c r="O33" s="12" t="n"/>
       <c r="P33" s="13">
         <f>I33+J33+K33+L33+M33+N33+O33</f>
         <v/>
@@ -3290,27 +2898,13 @@
         <f>D34+E34+F34+G34</f>
         <v/>
       </c>
-      <c r="I34" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J34" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K34" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L34" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M34" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N34" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O34" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I34" s="12" t="n"/>
+      <c r="J34" s="12" t="n"/>
+      <c r="K34" s="12" t="n"/>
+      <c r="L34" s="12" t="n"/>
+      <c r="M34" s="12" t="n"/>
+      <c r="N34" s="12" t="n"/>
+      <c r="O34" s="12" t="n"/>
       <c r="P34" s="13">
         <f>I34+J34+K34+L34+M34+N34+O34</f>
         <v/>
@@ -3368,27 +2962,13 @@
         <f>D35+E35+F35+G35</f>
         <v/>
       </c>
-      <c r="I35" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J35" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K35" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L35" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M35" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N35" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O35" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I35" s="12" t="n"/>
+      <c r="J35" s="12" t="n"/>
+      <c r="K35" s="12" t="n"/>
+      <c r="L35" s="12" t="n"/>
+      <c r="M35" s="12" t="n"/>
+      <c r="N35" s="12" t="n"/>
+      <c r="O35" s="12" t="n"/>
       <c r="P35" s="13">
         <f>I35+J35+K35+L35+M35+N35+O35</f>
         <v/>
@@ -3446,27 +3026,13 @@
         <f>D36+E36+F36+G36</f>
         <v/>
       </c>
-      <c r="I36" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J36" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K36" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L36" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M36" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N36" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O36" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I36" s="12" t="n"/>
+      <c r="J36" s="12" t="n"/>
+      <c r="K36" s="12" t="n"/>
+      <c r="L36" s="12" t="n"/>
+      <c r="M36" s="12" t="n"/>
+      <c r="N36" s="12" t="n"/>
+      <c r="O36" s="12" t="n"/>
       <c r="P36" s="13">
         <f>I36+J36+K36+L36+M36+N36+O36</f>
         <v/>
@@ -3524,27 +3090,13 @@
         <f>D37+E37+F37+G37</f>
         <v/>
       </c>
-      <c r="I37" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J37" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K37" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L37" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M37" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N37" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O37" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I37" s="12" t="n"/>
+      <c r="J37" s="12" t="n"/>
+      <c r="K37" s="12" t="n"/>
+      <c r="L37" s="12" t="n"/>
+      <c r="M37" s="12" t="n"/>
+      <c r="N37" s="12" t="n"/>
+      <c r="O37" s="12" t="n"/>
       <c r="P37" s="13">
         <f>I37+J37+K37+L37+M37+N37+O37</f>
         <v/>
@@ -3602,27 +3154,13 @@
         <f>D38+E38+F38+G38</f>
         <v/>
       </c>
-      <c r="I38" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J38" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K38" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L38" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M38" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N38" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O38" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I38" s="12" t="n"/>
+      <c r="J38" s="12" t="n"/>
+      <c r="K38" s="12" t="n"/>
+      <c r="L38" s="12" t="n"/>
+      <c r="M38" s="12" t="n"/>
+      <c r="N38" s="12" t="n"/>
+      <c r="O38" s="12" t="n"/>
       <c r="P38" s="13">
         <f>I38+J38+K38+L38+M38+N38+O38</f>
         <v/>
@@ -3680,27 +3218,13 @@
         <f>D39+E39+F39+G39</f>
         <v/>
       </c>
-      <c r="I39" s="12" t="n">
-        <v>430000</v>
-      </c>
-      <c r="J39" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="K39" s="12" t="n">
-        <v>67000</v>
-      </c>
-      <c r="L39" s="12" t="n">
-        <v>385000</v>
-      </c>
-      <c r="M39" s="12" t="n">
-        <v>43000</v>
-      </c>
-      <c r="N39" s="12" t="n">
-        <v>29000</v>
-      </c>
-      <c r="O39" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="I39" s="12" t="n"/>
+      <c r="J39" s="12" t="n"/>
+      <c r="K39" s="12" t="n"/>
+      <c r="L39" s="12" t="n"/>
+      <c r="M39" s="12" t="n"/>
+      <c r="N39" s="12" t="n"/>
+      <c r="O39" s="12" t="n"/>
       <c r="P39" s="13">
         <f>I39+J39+K39+L39+M39+N39+O39</f>
         <v/>
@@ -3780,27 +3304,13 @@
         <f>D41+E41+F41+G41</f>
         <v/>
       </c>
-      <c r="I41" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J41" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K41" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L41" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M41" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N41" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O41" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I41" s="12" t="n"/>
+      <c r="J41" s="12" t="n"/>
+      <c r="K41" s="12" t="n"/>
+      <c r="L41" s="12" t="n"/>
+      <c r="M41" s="12" t="n"/>
+      <c r="N41" s="12" t="n"/>
+      <c r="O41" s="12" t="n"/>
       <c r="P41" s="13">
         <f>I41+J41+K41+L41+M41+N41+O41</f>
         <v/>
@@ -3859,27 +3369,13 @@
         <f>D42+E42+F42+G42</f>
         <v/>
       </c>
-      <c r="I42" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J42" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K42" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L42" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M42" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N42" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O42" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I42" s="12" t="n"/>
+      <c r="J42" s="12" t="n"/>
+      <c r="K42" s="12" t="n"/>
+      <c r="L42" s="12" t="n"/>
+      <c r="M42" s="12" t="n"/>
+      <c r="N42" s="12" t="n"/>
+      <c r="O42" s="12" t="n"/>
       <c r="P42" s="13">
         <f>I42+J42+K42+L42+M42+N42+O42</f>
         <v/>
@@ -3937,27 +3433,13 @@
         <f>D43+E43+F43+G43</f>
         <v/>
       </c>
-      <c r="I43" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J43" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K43" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L43" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M43" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N43" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O43" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I43" s="12" t="n"/>
+      <c r="J43" s="12" t="n"/>
+      <c r="K43" s="12" t="n"/>
+      <c r="L43" s="12" t="n"/>
+      <c r="M43" s="12" t="n"/>
+      <c r="N43" s="12" t="n"/>
+      <c r="O43" s="12" t="n"/>
       <c r="P43" s="13">
         <f>I43+J43+K43+L43+M43+N43+O43</f>
         <v/>
@@ -4015,27 +3497,13 @@
         <f>D44+E44+F44+G44</f>
         <v/>
       </c>
-      <c r="I44" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J44" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K44" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L44" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M44" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N44" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O44" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I44" s="12" t="n"/>
+      <c r="J44" s="12" t="n"/>
+      <c r="K44" s="12" t="n"/>
+      <c r="L44" s="12" t="n"/>
+      <c r="M44" s="12" t="n"/>
+      <c r="N44" s="12" t="n"/>
+      <c r="O44" s="12" t="n"/>
       <c r="P44" s="13">
         <f>I44+J44+K44+L44+M44+N44+O44</f>
         <v/>
@@ -4093,27 +3561,13 @@
         <f>D45+E45+F45+G45</f>
         <v/>
       </c>
-      <c r="I45" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J45" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K45" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L45" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M45" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N45" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O45" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I45" s="12" t="n"/>
+      <c r="J45" s="12" t="n"/>
+      <c r="K45" s="12" t="n"/>
+      <c r="L45" s="12" t="n"/>
+      <c r="M45" s="12" t="n"/>
+      <c r="N45" s="12" t="n"/>
+      <c r="O45" s="12" t="n"/>
       <c r="P45" s="13">
         <f>I45+J45+K45+L45+M45+N45+O45</f>
         <v/>
@@ -4171,27 +3625,13 @@
         <f>D46+E46+F46+G46</f>
         <v/>
       </c>
-      <c r="I46" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J46" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K46" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L46" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M46" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N46" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O46" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I46" s="12" t="n"/>
+      <c r="J46" s="12" t="n"/>
+      <c r="K46" s="12" t="n"/>
+      <c r="L46" s="12" t="n"/>
+      <c r="M46" s="12" t="n"/>
+      <c r="N46" s="12" t="n"/>
+      <c r="O46" s="12" t="n"/>
       <c r="P46" s="13">
         <f>I46+J46+K46+L46+M46+N46+O46</f>
         <v/>
@@ -4249,27 +3689,13 @@
         <f>D47+E47+F47+G47</f>
         <v/>
       </c>
-      <c r="I47" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J47" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K47" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L47" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M47" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N47" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O47" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I47" s="12" t="n"/>
+      <c r="J47" s="12" t="n"/>
+      <c r="K47" s="12" t="n"/>
+      <c r="L47" s="12" t="n"/>
+      <c r="M47" s="12" t="n"/>
+      <c r="N47" s="12" t="n"/>
+      <c r="O47" s="12" t="n"/>
       <c r="P47" s="13">
         <f>I47+J47+K47+L47+M47+N47+O47</f>
         <v/>
@@ -4327,27 +3753,13 @@
         <f>D48+E48+F48+G48</f>
         <v/>
       </c>
-      <c r="I48" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J48" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K48" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L48" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M48" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N48" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O48" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I48" s="12" t="n"/>
+      <c r="J48" s="12" t="n"/>
+      <c r="K48" s="12" t="n"/>
+      <c r="L48" s="12" t="n"/>
+      <c r="M48" s="12" t="n"/>
+      <c r="N48" s="12" t="n"/>
+      <c r="O48" s="12" t="n"/>
       <c r="P48" s="13">
         <f>I48+J48+K48+L48+M48+N48+O48</f>
         <v/>
@@ -4405,27 +3817,13 @@
         <f>D49+E49+F49+G49</f>
         <v/>
       </c>
-      <c r="I49" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J49" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K49" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L49" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M49" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N49" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O49" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I49" s="12" t="n"/>
+      <c r="J49" s="12" t="n"/>
+      <c r="K49" s="12" t="n"/>
+      <c r="L49" s="12" t="n"/>
+      <c r="M49" s="12" t="n"/>
+      <c r="N49" s="12" t="n"/>
+      <c r="O49" s="12" t="n"/>
       <c r="P49" s="13">
         <f>I49+J49+K49+L49+M49+N49+O49</f>
         <v/>
@@ -4483,27 +3881,13 @@
         <f>D50+E50+F50+G50</f>
         <v/>
       </c>
-      <c r="I50" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J50" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K50" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L50" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M50" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N50" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O50" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I50" s="12" t="n"/>
+      <c r="J50" s="12" t="n"/>
+      <c r="K50" s="12" t="n"/>
+      <c r="L50" s="12" t="n"/>
+      <c r="M50" s="12" t="n"/>
+      <c r="N50" s="12" t="n"/>
+      <c r="O50" s="12" t="n"/>
       <c r="P50" s="13">
         <f>I50+J50+K50+L50+M50+N50+O50</f>
         <v/>
@@ -4561,27 +3945,13 @@
         <f>D51+E51+F51+G51</f>
         <v/>
       </c>
-      <c r="I51" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J51" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K51" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L51" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M51" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N51" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O51" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I51" s="12" t="n"/>
+      <c r="J51" s="12" t="n"/>
+      <c r="K51" s="12" t="n"/>
+      <c r="L51" s="12" t="n"/>
+      <c r="M51" s="12" t="n"/>
+      <c r="N51" s="12" t="n"/>
+      <c r="O51" s="12" t="n"/>
       <c r="P51" s="13">
         <f>I51+J51+K51+L51+M51+N51+O51</f>
         <v/>
@@ -4639,27 +4009,13 @@
         <f>D52+E52+F52+G52</f>
         <v/>
       </c>
-      <c r="I52" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J52" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K52" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L52" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M52" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N52" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O52" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I52" s="12" t="n"/>
+      <c r="J52" s="12" t="n"/>
+      <c r="K52" s="12" t="n"/>
+      <c r="L52" s="12" t="n"/>
+      <c r="M52" s="12" t="n"/>
+      <c r="N52" s="12" t="n"/>
+      <c r="O52" s="12" t="n"/>
       <c r="P52" s="13">
         <f>I52+J52+K52+L52+M52+N52+O52</f>
         <v/>
@@ -4717,27 +4073,13 @@
         <f>D53+E53+F53+G53</f>
         <v/>
       </c>
-      <c r="I53" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J53" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K53" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L53" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M53" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N53" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O53" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I53" s="12" t="n"/>
+      <c r="J53" s="12" t="n"/>
+      <c r="K53" s="12" t="n"/>
+      <c r="L53" s="12" t="n"/>
+      <c r="M53" s="12" t="n"/>
+      <c r="N53" s="12" t="n"/>
+      <c r="O53" s="12" t="n"/>
       <c r="P53" s="13">
         <f>I53+J53+K53+L53+M53+N53+O53</f>
         <v/>
@@ -4795,27 +4137,13 @@
         <f>D54+E54+F54+G54</f>
         <v/>
       </c>
-      <c r="I54" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J54" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K54" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L54" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M54" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N54" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O54" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I54" s="12" t="n"/>
+      <c r="J54" s="12" t="n"/>
+      <c r="K54" s="12" t="n"/>
+      <c r="L54" s="12" t="n"/>
+      <c r="M54" s="12" t="n"/>
+      <c r="N54" s="12" t="n"/>
+      <c r="O54" s="12" t="n"/>
       <c r="P54" s="13">
         <f>I54+J54+K54+L54+M54+N54+O54</f>
         <v/>
@@ -4873,27 +4201,13 @@
         <f>D55+E55+F55+G55</f>
         <v/>
       </c>
-      <c r="I55" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J55" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K55" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L55" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M55" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N55" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O55" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I55" s="12" t="n"/>
+      <c r="J55" s="12" t="n"/>
+      <c r="K55" s="12" t="n"/>
+      <c r="L55" s="12" t="n"/>
+      <c r="M55" s="12" t="n"/>
+      <c r="N55" s="12" t="n"/>
+      <c r="O55" s="12" t="n"/>
       <c r="P55" s="13">
         <f>I55+J55+K55+L55+M55+N55+O55</f>
         <v/>
@@ -4951,27 +4265,13 @@
         <f>D56+E56+F56+G56</f>
         <v/>
       </c>
-      <c r="I56" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J56" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K56" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L56" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M56" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N56" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O56" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I56" s="12" t="n"/>
+      <c r="J56" s="12" t="n"/>
+      <c r="K56" s="12" t="n"/>
+      <c r="L56" s="12" t="n"/>
+      <c r="M56" s="12" t="n"/>
+      <c r="N56" s="12" t="n"/>
+      <c r="O56" s="12" t="n"/>
       <c r="P56" s="13">
         <f>I56+J56+K56+L56+M56+N56+O56</f>
         <v/>
@@ -5029,27 +4329,13 @@
         <f>D57+E57+F57+G57</f>
         <v/>
       </c>
-      <c r="I57" s="12" t="n">
-        <v>1360000</v>
-      </c>
-      <c r="J57" s="12" t="n">
-        <v>490000</v>
-      </c>
-      <c r="K57" s="12" t="n">
-        <v>220000</v>
-      </c>
-      <c r="L57" s="12" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="M57" s="12" t="n">
-        <v>165000</v>
-      </c>
-      <c r="N57" s="12" t="n">
-        <v>84000</v>
-      </c>
-      <c r="O57" s="12" t="n">
-        <v>210000</v>
-      </c>
+      <c r="I57" s="12" t="n"/>
+      <c r="J57" s="12" t="n"/>
+      <c r="K57" s="12" t="n"/>
+      <c r="L57" s="12" t="n"/>
+      <c r="M57" s="12" t="n"/>
+      <c r="N57" s="12" t="n"/>
+      <c r="O57" s="12" t="n"/>
       <c r="P57" s="13">
         <f>I57+J57+K57+L57+M57+N57+O57</f>
         <v/>

</xml_diff>

<commit_message>
Clear dummy cost values from ルート別採算 yellow input cells
Leave cost columns (人件費/燃料費/車両費/処理費/運搬費/その他) blank
so users can enter actual figures rather than seeing misleading estimates.

https://claude.ai/code/session_01BgHAFjDQSmbvXBnKUF79fq
</commit_message>
<xml_diff>
--- a/sacure_採算管理_v4_ルート別案件別.xlsx
+++ b/sacure_採算管理_v4_ルート別案件別.xlsx
@@ -5352,22 +5352,12 @@
         <f>IFERROR(VLOOKUP(C5,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E5" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F5" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G5" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E5" s="12" t="n"/>
+      <c r="F5" s="12" t="n"/>
+      <c r="G5" s="12" t="n"/>
       <c r="H5" s="12" t="n"/>
-      <c r="I5" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I5" s="12" t="n"/>
+      <c r="J5" s="12" t="n"/>
       <c r="K5" s="13">
         <f>E5+F5+G5+H5+I5+J5</f>
         <v/>
@@ -5419,22 +5409,12 @@
         <f>IFERROR(VLOOKUP(C6,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E6" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F6" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G6" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E6" s="12" t="n"/>
+      <c r="F6" s="12" t="n"/>
+      <c r="G6" s="12" t="n"/>
       <c r="H6" s="12" t="n"/>
-      <c r="I6" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I6" s="12" t="n"/>
+      <c r="J6" s="12" t="n"/>
       <c r="K6" s="13">
         <f>E6+F6+G6+H6+I6+J6</f>
         <v/>
@@ -5485,22 +5465,12 @@
         <f>IFERROR(VLOOKUP(C7,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E7" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F7" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G7" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E7" s="12" t="n"/>
+      <c r="F7" s="12" t="n"/>
+      <c r="G7" s="12" t="n"/>
       <c r="H7" s="12" t="n"/>
-      <c r="I7" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J7" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="12" t="n"/>
       <c r="K7" s="13">
         <f>E7+F7+G7+H7+I7+J7</f>
         <v/>
@@ -5551,22 +5521,12 @@
         <f>IFERROR(VLOOKUP(C8,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E8" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G8" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
       <c r="H8" s="12" t="n"/>
-      <c r="I8" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J8" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
       <c r="K8" s="13">
         <f>E8+F8+G8+H8+I8+J8</f>
         <v/>
@@ -5617,22 +5577,12 @@
         <f>IFERROR(VLOOKUP(C9,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E9" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F9" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G9" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
       <c r="H9" s="12" t="n"/>
-      <c r="I9" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="12" t="n"/>
       <c r="K9" s="13">
         <f>E9+F9+G9+H9+I9+J9</f>
         <v/>
@@ -5683,22 +5633,12 @@
         <f>IFERROR(VLOOKUP(C10,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E10" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F10" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G10" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="12" t="n"/>
       <c r="H10" s="12" t="n"/>
-      <c r="I10" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="12" t="n"/>
       <c r="K10" s="13">
         <f>E10+F10+G10+H10+I10+J10</f>
         <v/>
@@ -5749,22 +5689,12 @@
         <f>IFERROR(VLOOKUP(C11,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E11" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F11" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G11" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
       <c r="H11" s="12" t="n"/>
-      <c r="I11" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="n"/>
       <c r="K11" s="13">
         <f>E11+F11+G11+H11+I11+J11</f>
         <v/>
@@ -5815,22 +5745,12 @@
         <f>IFERROR(VLOOKUP(C12,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E12" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G12" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
       <c r="H12" s="12" t="n"/>
-      <c r="I12" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="12" t="n"/>
       <c r="K12" s="13">
         <f>E12+F12+G12+H12+I12+J12</f>
         <v/>
@@ -5881,22 +5801,12 @@
         <f>IFERROR(VLOOKUP(C13,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E13" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F13" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G13" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
       <c r="H13" s="12" t="n"/>
-      <c r="I13" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J13" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="12" t="n"/>
       <c r="K13" s="13">
         <f>E13+F13+G13+H13+I13+J13</f>
         <v/>
@@ -5947,22 +5857,12 @@
         <f>IFERROR(VLOOKUP(C14,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E14" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F14" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G14" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="12" t="n"/>
       <c r="H14" s="12" t="n"/>
-      <c r="I14" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J14" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I14" s="12" t="n"/>
+      <c r="J14" s="12" t="n"/>
       <c r="K14" s="13">
         <f>E14+F14+G14+H14+I14+J14</f>
         <v/>
@@ -6013,22 +5913,12 @@
         <f>IFERROR(VLOOKUP(C15,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E15" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F15" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G15" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="12" t="n"/>
+      <c r="G15" s="12" t="n"/>
       <c r="H15" s="12" t="n"/>
-      <c r="I15" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I15" s="12" t="n"/>
+      <c r="J15" s="12" t="n"/>
       <c r="K15" s="13">
         <f>E15+F15+G15+H15+I15+J15</f>
         <v/>
@@ -6079,22 +5969,12 @@
         <f>IFERROR(VLOOKUP(C16,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E16" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F16" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G16" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="12" t="n"/>
       <c r="H16" s="12" t="n"/>
-      <c r="I16" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I16" s="12" t="n"/>
+      <c r="J16" s="12" t="n"/>
       <c r="K16" s="13">
         <f>E16+F16+G16+H16+I16+J16</f>
         <v/>
@@ -6145,22 +6025,12 @@
         <f>IFERROR(VLOOKUP(C17,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E17" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F17" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G17" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
       <c r="H17" s="12" t="n"/>
-      <c r="I17" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="12" t="n"/>
       <c r="K17" s="13">
         <f>E17+F17+G17+H17+I17+J17</f>
         <v/>
@@ -6211,22 +6081,12 @@
         <f>IFERROR(VLOOKUP(C18,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E18" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F18" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G18" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="12" t="n"/>
       <c r="H18" s="12" t="n"/>
-      <c r="I18" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I18" s="12" t="n"/>
+      <c r="J18" s="12" t="n"/>
       <c r="K18" s="13">
         <f>E18+F18+G18+H18+I18+J18</f>
         <v/>
@@ -6277,22 +6137,12 @@
         <f>IFERROR(VLOOKUP(C19,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E19" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F19" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G19" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="12" t="n"/>
       <c r="H19" s="12" t="n"/>
-      <c r="I19" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J19" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I19" s="12" t="n"/>
+      <c r="J19" s="12" t="n"/>
       <c r="K19" s="13">
         <f>E19+F19+G19+H19+I19+J19</f>
         <v/>
@@ -6343,22 +6193,12 @@
         <f>IFERROR(VLOOKUP(C20,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E20" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F20" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G20" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="12" t="n"/>
       <c r="H20" s="12" t="n"/>
-      <c r="I20" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J20" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I20" s="12" t="n"/>
+      <c r="J20" s="12" t="n"/>
       <c r="K20" s="13">
         <f>E20+F20+G20+H20+I20+J20</f>
         <v/>
@@ -6409,22 +6249,12 @@
         <f>IFERROR(VLOOKUP(C21,▼売上原票!$A:$P,3,0),0)</f>
         <v/>
       </c>
-      <c r="E21" s="12" t="n">
-        <v>650000</v>
-      </c>
-      <c r="F21" s="12" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G21" s="12" t="n">
-        <v>85000</v>
-      </c>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="12" t="n"/>
       <c r="H21" s="12" t="n"/>
-      <c r="I21" s="12" t="n">
-        <v>75000</v>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>45000</v>
-      </c>
+      <c r="I21" s="12" t="n"/>
+      <c r="J21" s="12" t="n"/>
       <c r="K21" s="13">
         <f>E21+F21+G21+H21+I21+J21</f>
         <v/>
@@ -6494,24 +6324,12 @@
         <f>IFERROR(VLOOKUP(C23,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E23" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F23" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G23" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H23" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I23" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="12" t="n"/>
+      <c r="J23" s="12" t="n"/>
       <c r="K23" s="13">
         <f>E23+F23+G23+H23+I23+J23</f>
         <v/>
@@ -6563,24 +6381,12 @@
         <f>IFERROR(VLOOKUP(C24,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E24" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F24" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G24" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H24" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I24" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J24" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="12" t="n"/>
+      <c r="H24" s="12" t="n"/>
+      <c r="I24" s="12" t="n"/>
+      <c r="J24" s="12" t="n"/>
       <c r="K24" s="13">
         <f>E24+F24+G24+H24+I24+J24</f>
         <v/>
@@ -6631,24 +6437,12 @@
         <f>IFERROR(VLOOKUP(C25,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E25" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F25" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G25" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H25" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I25" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J25" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="12" t="n"/>
+      <c r="I25" s="12" t="n"/>
+      <c r="J25" s="12" t="n"/>
       <c r="K25" s="13">
         <f>E25+F25+G25+H25+I25+J25</f>
         <v/>
@@ -6699,24 +6493,12 @@
         <f>IFERROR(VLOOKUP(C26,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E26" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F26" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G26" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H26" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I26" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J26" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E26" s="12" t="n"/>
+      <c r="F26" s="12" t="n"/>
+      <c r="G26" s="12" t="n"/>
+      <c r="H26" s="12" t="n"/>
+      <c r="I26" s="12" t="n"/>
+      <c r="J26" s="12" t="n"/>
       <c r="K26" s="13">
         <f>E26+F26+G26+H26+I26+J26</f>
         <v/>
@@ -6767,24 +6549,12 @@
         <f>IFERROR(VLOOKUP(C27,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E27" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F27" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G27" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H27" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I27" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J27" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="12" t="n"/>
+      <c r="J27" s="12" t="n"/>
       <c r="K27" s="13">
         <f>E27+F27+G27+H27+I27+J27</f>
         <v/>
@@ -6835,24 +6605,12 @@
         <f>IFERROR(VLOOKUP(C28,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E28" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F28" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G28" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H28" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I28" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J28" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="12" t="n"/>
+      <c r="H28" s="12" t="n"/>
+      <c r="I28" s="12" t="n"/>
+      <c r="J28" s="12" t="n"/>
       <c r="K28" s="13">
         <f>E28+F28+G28+H28+I28+J28</f>
         <v/>
@@ -6903,24 +6661,12 @@
         <f>IFERROR(VLOOKUP(C29,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E29" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F29" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G29" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H29" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I29" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J29" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="12" t="n"/>
+      <c r="H29" s="12" t="n"/>
+      <c r="I29" s="12" t="n"/>
+      <c r="J29" s="12" t="n"/>
       <c r="K29" s="13">
         <f>E29+F29+G29+H29+I29+J29</f>
         <v/>
@@ -6971,24 +6717,12 @@
         <f>IFERROR(VLOOKUP(C30,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E30" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F30" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G30" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H30" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I30" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J30" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="12" t="n"/>
+      <c r="G30" s="12" t="n"/>
+      <c r="H30" s="12" t="n"/>
+      <c r="I30" s="12" t="n"/>
+      <c r="J30" s="12" t="n"/>
       <c r="K30" s="13">
         <f>E30+F30+G30+H30+I30+J30</f>
         <v/>
@@ -7039,24 +6773,12 @@
         <f>IFERROR(VLOOKUP(C31,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E31" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F31" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G31" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H31" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I31" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J31" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+      <c r="I31" s="12" t="n"/>
+      <c r="J31" s="12" t="n"/>
       <c r="K31" s="13">
         <f>E31+F31+G31+H31+I31+J31</f>
         <v/>
@@ -7107,24 +6829,12 @@
         <f>IFERROR(VLOOKUP(C32,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E32" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F32" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G32" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H32" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I32" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J32" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E32" s="12" t="n"/>
+      <c r="F32" s="12" t="n"/>
+      <c r="G32" s="12" t="n"/>
+      <c r="H32" s="12" t="n"/>
+      <c r="I32" s="12" t="n"/>
+      <c r="J32" s="12" t="n"/>
       <c r="K32" s="13">
         <f>E32+F32+G32+H32+I32+J32</f>
         <v/>
@@ -7175,24 +6885,12 @@
         <f>IFERROR(VLOOKUP(C33,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E33" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F33" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G33" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H33" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I33" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J33" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="12" t="n"/>
+      <c r="G33" s="12" t="n"/>
+      <c r="H33" s="12" t="n"/>
+      <c r="I33" s="12" t="n"/>
+      <c r="J33" s="12" t="n"/>
       <c r="K33" s="13">
         <f>E33+F33+G33+H33+I33+J33</f>
         <v/>
@@ -7243,24 +6941,12 @@
         <f>IFERROR(VLOOKUP(C34,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E34" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F34" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G34" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H34" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I34" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J34" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E34" s="12" t="n"/>
+      <c r="F34" s="12" t="n"/>
+      <c r="G34" s="12" t="n"/>
+      <c r="H34" s="12" t="n"/>
+      <c r="I34" s="12" t="n"/>
+      <c r="J34" s="12" t="n"/>
       <c r="K34" s="13">
         <f>E34+F34+G34+H34+I34+J34</f>
         <v/>
@@ -7311,24 +6997,12 @@
         <f>IFERROR(VLOOKUP(C35,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E35" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F35" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G35" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H35" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I35" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J35" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="12" t="n"/>
+      <c r="G35" s="12" t="n"/>
+      <c r="H35" s="12" t="n"/>
+      <c r="I35" s="12" t="n"/>
+      <c r="J35" s="12" t="n"/>
       <c r="K35" s="13">
         <f>E35+F35+G35+H35+I35+J35</f>
         <v/>
@@ -7379,24 +7053,12 @@
         <f>IFERROR(VLOOKUP(C36,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E36" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F36" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G36" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H36" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I36" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J36" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E36" s="12" t="n"/>
+      <c r="F36" s="12" t="n"/>
+      <c r="G36" s="12" t="n"/>
+      <c r="H36" s="12" t="n"/>
+      <c r="I36" s="12" t="n"/>
+      <c r="J36" s="12" t="n"/>
       <c r="K36" s="13">
         <f>E36+F36+G36+H36+I36+J36</f>
         <v/>
@@ -7447,24 +7109,12 @@
         <f>IFERROR(VLOOKUP(C37,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E37" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F37" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G37" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H37" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I37" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J37" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E37" s="12" t="n"/>
+      <c r="F37" s="12" t="n"/>
+      <c r="G37" s="12" t="n"/>
+      <c r="H37" s="12" t="n"/>
+      <c r="I37" s="12" t="n"/>
+      <c r="J37" s="12" t="n"/>
       <c r="K37" s="13">
         <f>E37+F37+G37+H37+I37+J37</f>
         <v/>
@@ -7515,24 +7165,12 @@
         <f>IFERROR(VLOOKUP(C38,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E38" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F38" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G38" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H38" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I38" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J38" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="12" t="n"/>
+      <c r="G38" s="12" t="n"/>
+      <c r="H38" s="12" t="n"/>
+      <c r="I38" s="12" t="n"/>
+      <c r="J38" s="12" t="n"/>
       <c r="K38" s="13">
         <f>E38+F38+G38+H38+I38+J38</f>
         <v/>
@@ -7583,24 +7221,12 @@
         <f>IFERROR(VLOOKUP(C39,▼売上原票!$A:$P,4,0),0)</f>
         <v/>
       </c>
-      <c r="E39" s="12" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F39" s="12" t="n">
-        <v>520000</v>
-      </c>
-      <c r="G39" s="12" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H39" s="12" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="I39" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="J39" s="12" t="n">
-        <v>120000</v>
-      </c>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="12" t="n"/>
+      <c r="G39" s="12" t="n"/>
+      <c r="H39" s="12" t="n"/>
+      <c r="I39" s="12" t="n"/>
+      <c r="J39" s="12" t="n"/>
       <c r="K39" s="13">
         <f>E39+F39+G39+H39+I39+J39</f>
         <v/>
@@ -7670,22 +7296,12 @@
         <f>IFERROR(VLOOKUP(C41,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E41" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F41" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G41" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E41" s="12" t="n"/>
+      <c r="F41" s="12" t="n"/>
+      <c r="G41" s="12" t="n"/>
       <c r="H41" s="12" t="n"/>
-      <c r="I41" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J41" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I41" s="12" t="n"/>
+      <c r="J41" s="12" t="n"/>
       <c r="K41" s="13">
         <f>E41+F41+G41+H41+I41+J41</f>
         <v/>
@@ -7737,22 +7353,12 @@
         <f>IFERROR(VLOOKUP(C42,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E42" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F42" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G42" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="12" t="n"/>
+      <c r="G42" s="12" t="n"/>
       <c r="H42" s="12" t="n"/>
-      <c r="I42" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J42" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I42" s="12" t="n"/>
+      <c r="J42" s="12" t="n"/>
       <c r="K42" s="13">
         <f>E42+F42+G42+H42+I42+J42</f>
         <v/>
@@ -7803,22 +7409,12 @@
         <f>IFERROR(VLOOKUP(C43,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E43" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F43" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G43" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E43" s="12" t="n"/>
+      <c r="F43" s="12" t="n"/>
+      <c r="G43" s="12" t="n"/>
       <c r="H43" s="12" t="n"/>
-      <c r="I43" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J43" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I43" s="12" t="n"/>
+      <c r="J43" s="12" t="n"/>
       <c r="K43" s="13">
         <f>E43+F43+G43+H43+I43+J43</f>
         <v/>
@@ -7869,22 +7465,12 @@
         <f>IFERROR(VLOOKUP(C44,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E44" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F44" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G44" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="12" t="n"/>
+      <c r="G44" s="12" t="n"/>
       <c r="H44" s="12" t="n"/>
-      <c r="I44" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J44" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I44" s="12" t="n"/>
+      <c r="J44" s="12" t="n"/>
       <c r="K44" s="13">
         <f>E44+F44+G44+H44+I44+J44</f>
         <v/>
@@ -7935,22 +7521,12 @@
         <f>IFERROR(VLOOKUP(C45,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E45" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F45" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G45" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="12" t="n"/>
+      <c r="G45" s="12" t="n"/>
       <c r="H45" s="12" t="n"/>
-      <c r="I45" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J45" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I45" s="12" t="n"/>
+      <c r="J45" s="12" t="n"/>
       <c r="K45" s="13">
         <f>E45+F45+G45+H45+I45+J45</f>
         <v/>
@@ -8001,22 +7577,12 @@
         <f>IFERROR(VLOOKUP(C46,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E46" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F46" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G46" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E46" s="12" t="n"/>
+      <c r="F46" s="12" t="n"/>
+      <c r="G46" s="12" t="n"/>
       <c r="H46" s="12" t="n"/>
-      <c r="I46" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J46" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I46" s="12" t="n"/>
+      <c r="J46" s="12" t="n"/>
       <c r="K46" s="13">
         <f>E46+F46+G46+H46+I46+J46</f>
         <v/>
@@ -8067,22 +7633,12 @@
         <f>IFERROR(VLOOKUP(C47,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E47" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F47" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G47" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="12" t="n"/>
+      <c r="G47" s="12" t="n"/>
       <c r="H47" s="12" t="n"/>
-      <c r="I47" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J47" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I47" s="12" t="n"/>
+      <c r="J47" s="12" t="n"/>
       <c r="K47" s="13">
         <f>E47+F47+G47+H47+I47+J47</f>
         <v/>
@@ -8133,22 +7689,12 @@
         <f>IFERROR(VLOOKUP(C48,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E48" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F48" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G48" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E48" s="12" t="n"/>
+      <c r="F48" s="12" t="n"/>
+      <c r="G48" s="12" t="n"/>
       <c r="H48" s="12" t="n"/>
-      <c r="I48" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J48" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I48" s="12" t="n"/>
+      <c r="J48" s="12" t="n"/>
       <c r="K48" s="13">
         <f>E48+F48+G48+H48+I48+J48</f>
         <v/>
@@ -8199,22 +7745,12 @@
         <f>IFERROR(VLOOKUP(C49,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E49" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F49" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G49" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E49" s="12" t="n"/>
+      <c r="F49" s="12" t="n"/>
+      <c r="G49" s="12" t="n"/>
       <c r="H49" s="12" t="n"/>
-      <c r="I49" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J49" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I49" s="12" t="n"/>
+      <c r="J49" s="12" t="n"/>
       <c r="K49" s="13">
         <f>E49+F49+G49+H49+I49+J49</f>
         <v/>
@@ -8265,22 +7801,12 @@
         <f>IFERROR(VLOOKUP(C50,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E50" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F50" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G50" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E50" s="12" t="n"/>
+      <c r="F50" s="12" t="n"/>
+      <c r="G50" s="12" t="n"/>
       <c r="H50" s="12" t="n"/>
-      <c r="I50" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J50" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I50" s="12" t="n"/>
+      <c r="J50" s="12" t="n"/>
       <c r="K50" s="13">
         <f>E50+F50+G50+H50+I50+J50</f>
         <v/>
@@ -8331,22 +7857,12 @@
         <f>IFERROR(VLOOKUP(C51,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E51" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F51" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G51" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E51" s="12" t="n"/>
+      <c r="F51" s="12" t="n"/>
+      <c r="G51" s="12" t="n"/>
       <c r="H51" s="12" t="n"/>
-      <c r="I51" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J51" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I51" s="12" t="n"/>
+      <c r="J51" s="12" t="n"/>
       <c r="K51" s="13">
         <f>E51+F51+G51+H51+I51+J51</f>
         <v/>
@@ -8397,22 +7913,12 @@
         <f>IFERROR(VLOOKUP(C52,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E52" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F52" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G52" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E52" s="12" t="n"/>
+      <c r="F52" s="12" t="n"/>
+      <c r="G52" s="12" t="n"/>
       <c r="H52" s="12" t="n"/>
-      <c r="I52" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J52" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I52" s="12" t="n"/>
+      <c r="J52" s="12" t="n"/>
       <c r="K52" s="13">
         <f>E52+F52+G52+H52+I52+J52</f>
         <v/>
@@ -8463,22 +7969,12 @@
         <f>IFERROR(VLOOKUP(C53,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E53" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F53" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G53" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E53" s="12" t="n"/>
+      <c r="F53" s="12" t="n"/>
+      <c r="G53" s="12" t="n"/>
       <c r="H53" s="12" t="n"/>
-      <c r="I53" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J53" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I53" s="12" t="n"/>
+      <c r="J53" s="12" t="n"/>
       <c r="K53" s="13">
         <f>E53+F53+G53+H53+I53+J53</f>
         <v/>
@@ -8529,22 +8025,12 @@
         <f>IFERROR(VLOOKUP(C54,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E54" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F54" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G54" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E54" s="12" t="n"/>
+      <c r="F54" s="12" t="n"/>
+      <c r="G54" s="12" t="n"/>
       <c r="H54" s="12" t="n"/>
-      <c r="I54" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J54" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I54" s="12" t="n"/>
+      <c r="J54" s="12" t="n"/>
       <c r="K54" s="13">
         <f>E54+F54+G54+H54+I54+J54</f>
         <v/>
@@ -8595,22 +8081,12 @@
         <f>IFERROR(VLOOKUP(C55,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E55" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F55" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G55" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E55" s="12" t="n"/>
+      <c r="F55" s="12" t="n"/>
+      <c r="G55" s="12" t="n"/>
       <c r="H55" s="12" t="n"/>
-      <c r="I55" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J55" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I55" s="12" t="n"/>
+      <c r="J55" s="12" t="n"/>
       <c r="K55" s="13">
         <f>E55+F55+G55+H55+I55+J55</f>
         <v/>
@@ -8661,22 +8137,12 @@
         <f>IFERROR(VLOOKUP(C56,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E56" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F56" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G56" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E56" s="12" t="n"/>
+      <c r="F56" s="12" t="n"/>
+      <c r="G56" s="12" t="n"/>
       <c r="H56" s="12" t="n"/>
-      <c r="I56" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J56" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I56" s="12" t="n"/>
+      <c r="J56" s="12" t="n"/>
       <c r="K56" s="13">
         <f>E56+F56+G56+H56+I56+J56</f>
         <v/>
@@ -8727,22 +8193,12 @@
         <f>IFERROR(VLOOKUP(C57,▼売上原票!$A:$P,5,0),0)</f>
         <v/>
       </c>
-      <c r="E57" s="12" t="n">
-        <v>180000</v>
-      </c>
-      <c r="F57" s="12" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G57" s="12" t="n">
-        <v>180000</v>
-      </c>
+      <c r="E57" s="12" t="n"/>
+      <c r="F57" s="12" t="n"/>
+      <c r="G57" s="12" t="n"/>
       <c r="H57" s="12" t="n"/>
-      <c r="I57" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="J57" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="I57" s="12" t="n"/>
+      <c r="J57" s="12" t="n"/>
       <c r="K57" s="13">
         <f>E57+F57+G57+H57+I57+J57</f>
         <v/>
@@ -9784,22 +9240,12 @@
         <f>IFERROR(VLOOKUP(C77,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E77" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F77" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G77" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E77" s="12" t="n"/>
+      <c r="F77" s="12" t="n"/>
+      <c r="G77" s="12" t="n"/>
       <c r="H77" s="12" t="n"/>
-      <c r="I77" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J77" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I77" s="12" t="n"/>
+      <c r="J77" s="12" t="n"/>
       <c r="K77" s="13">
         <f>E77+F77+G77+H77+I77+J77</f>
         <v/>
@@ -9851,22 +9297,12 @@
         <f>IFERROR(VLOOKUP(C78,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E78" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F78" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G78" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E78" s="12" t="n"/>
+      <c r="F78" s="12" t="n"/>
+      <c r="G78" s="12" t="n"/>
       <c r="H78" s="12" t="n"/>
-      <c r="I78" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J78" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I78" s="12" t="n"/>
+      <c r="J78" s="12" t="n"/>
       <c r="K78" s="13">
         <f>E78+F78+G78+H78+I78+J78</f>
         <v/>
@@ -9917,22 +9353,12 @@
         <f>IFERROR(VLOOKUP(C79,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E79" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F79" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G79" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E79" s="12" t="n"/>
+      <c r="F79" s="12" t="n"/>
+      <c r="G79" s="12" t="n"/>
       <c r="H79" s="12" t="n"/>
-      <c r="I79" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J79" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I79" s="12" t="n"/>
+      <c r="J79" s="12" t="n"/>
       <c r="K79" s="13">
         <f>E79+F79+G79+H79+I79+J79</f>
         <v/>
@@ -9983,22 +9409,12 @@
         <f>IFERROR(VLOOKUP(C80,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E80" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F80" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G80" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E80" s="12" t="n"/>
+      <c r="F80" s="12" t="n"/>
+      <c r="G80" s="12" t="n"/>
       <c r="H80" s="12" t="n"/>
-      <c r="I80" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J80" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I80" s="12" t="n"/>
+      <c r="J80" s="12" t="n"/>
       <c r="K80" s="13">
         <f>E80+F80+G80+H80+I80+J80</f>
         <v/>
@@ -10049,22 +9465,12 @@
         <f>IFERROR(VLOOKUP(C81,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E81" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F81" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G81" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E81" s="12" t="n"/>
+      <c r="F81" s="12" t="n"/>
+      <c r="G81" s="12" t="n"/>
       <c r="H81" s="12" t="n"/>
-      <c r="I81" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J81" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I81" s="12" t="n"/>
+      <c r="J81" s="12" t="n"/>
       <c r="K81" s="13">
         <f>E81+F81+G81+H81+I81+J81</f>
         <v/>
@@ -10115,22 +9521,12 @@
         <f>IFERROR(VLOOKUP(C82,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E82" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F82" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G82" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E82" s="12" t="n"/>
+      <c r="F82" s="12" t="n"/>
+      <c r="G82" s="12" t="n"/>
       <c r="H82" s="12" t="n"/>
-      <c r="I82" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J82" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I82" s="12" t="n"/>
+      <c r="J82" s="12" t="n"/>
       <c r="K82" s="13">
         <f>E82+F82+G82+H82+I82+J82</f>
         <v/>
@@ -10181,22 +9577,12 @@
         <f>IFERROR(VLOOKUP(C83,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E83" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F83" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G83" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E83" s="12" t="n"/>
+      <c r="F83" s="12" t="n"/>
+      <c r="G83" s="12" t="n"/>
       <c r="H83" s="12" t="n"/>
-      <c r="I83" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J83" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I83" s="12" t="n"/>
+      <c r="J83" s="12" t="n"/>
       <c r="K83" s="13">
         <f>E83+F83+G83+H83+I83+J83</f>
         <v/>
@@ -10247,22 +9633,12 @@
         <f>IFERROR(VLOOKUP(C84,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E84" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F84" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G84" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E84" s="12" t="n"/>
+      <c r="F84" s="12" t="n"/>
+      <c r="G84" s="12" t="n"/>
       <c r="H84" s="12" t="n"/>
-      <c r="I84" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J84" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I84" s="12" t="n"/>
+      <c r="J84" s="12" t="n"/>
       <c r="K84" s="13">
         <f>E84+F84+G84+H84+I84+J84</f>
         <v/>
@@ -10313,22 +9689,12 @@
         <f>IFERROR(VLOOKUP(C85,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E85" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F85" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G85" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E85" s="12" t="n"/>
+      <c r="F85" s="12" t="n"/>
+      <c r="G85" s="12" t="n"/>
       <c r="H85" s="12" t="n"/>
-      <c r="I85" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J85" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I85" s="12" t="n"/>
+      <c r="J85" s="12" t="n"/>
       <c r="K85" s="13">
         <f>E85+F85+G85+H85+I85+J85</f>
         <v/>
@@ -10379,22 +9745,12 @@
         <f>IFERROR(VLOOKUP(C86,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E86" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F86" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G86" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E86" s="12" t="n"/>
+      <c r="F86" s="12" t="n"/>
+      <c r="G86" s="12" t="n"/>
       <c r="H86" s="12" t="n"/>
-      <c r="I86" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J86" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I86" s="12" t="n"/>
+      <c r="J86" s="12" t="n"/>
       <c r="K86" s="13">
         <f>E86+F86+G86+H86+I86+J86</f>
         <v/>
@@ -10445,22 +9801,12 @@
         <f>IFERROR(VLOOKUP(C87,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E87" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F87" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G87" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E87" s="12" t="n"/>
+      <c r="F87" s="12" t="n"/>
+      <c r="G87" s="12" t="n"/>
       <c r="H87" s="12" t="n"/>
-      <c r="I87" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J87" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I87" s="12" t="n"/>
+      <c r="J87" s="12" t="n"/>
       <c r="K87" s="13">
         <f>E87+F87+G87+H87+I87+J87</f>
         <v/>
@@ -10511,22 +9857,12 @@
         <f>IFERROR(VLOOKUP(C88,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E88" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F88" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G88" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E88" s="12" t="n"/>
+      <c r="F88" s="12" t="n"/>
+      <c r="G88" s="12" t="n"/>
       <c r="H88" s="12" t="n"/>
-      <c r="I88" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J88" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I88" s="12" t="n"/>
+      <c r="J88" s="12" t="n"/>
       <c r="K88" s="13">
         <f>E88+F88+G88+H88+I88+J88</f>
         <v/>
@@ -10577,22 +9913,12 @@
         <f>IFERROR(VLOOKUP(C89,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E89" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F89" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G89" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E89" s="12" t="n"/>
+      <c r="F89" s="12" t="n"/>
+      <c r="G89" s="12" t="n"/>
       <c r="H89" s="12" t="n"/>
-      <c r="I89" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J89" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I89" s="12" t="n"/>
+      <c r="J89" s="12" t="n"/>
       <c r="K89" s="13">
         <f>E89+F89+G89+H89+I89+J89</f>
         <v/>
@@ -10643,22 +9969,12 @@
         <f>IFERROR(VLOOKUP(C90,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E90" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F90" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G90" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E90" s="12" t="n"/>
+      <c r="F90" s="12" t="n"/>
+      <c r="G90" s="12" t="n"/>
       <c r="H90" s="12" t="n"/>
-      <c r="I90" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J90" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I90" s="12" t="n"/>
+      <c r="J90" s="12" t="n"/>
       <c r="K90" s="13">
         <f>E90+F90+G90+H90+I90+J90</f>
         <v/>
@@ -10709,22 +10025,12 @@
         <f>IFERROR(VLOOKUP(C91,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E91" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F91" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G91" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E91" s="12" t="n"/>
+      <c r="F91" s="12" t="n"/>
+      <c r="G91" s="12" t="n"/>
       <c r="H91" s="12" t="n"/>
-      <c r="I91" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J91" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I91" s="12" t="n"/>
+      <c r="J91" s="12" t="n"/>
       <c r="K91" s="13">
         <f>E91+F91+G91+H91+I91+J91</f>
         <v/>
@@ -10775,22 +10081,12 @@
         <f>IFERROR(VLOOKUP(C92,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E92" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F92" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G92" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E92" s="12" t="n"/>
+      <c r="F92" s="12" t="n"/>
+      <c r="G92" s="12" t="n"/>
       <c r="H92" s="12" t="n"/>
-      <c r="I92" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J92" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I92" s="12" t="n"/>
+      <c r="J92" s="12" t="n"/>
       <c r="K92" s="13">
         <f>E92+F92+G92+H92+I92+J92</f>
         <v/>
@@ -10841,22 +10137,12 @@
         <f>IFERROR(VLOOKUP(C93,▼売上原票!$A:$P,7,0),0)</f>
         <v/>
       </c>
-      <c r="E93" s="12" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F93" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G93" s="12" t="n">
-        <v>15000</v>
-      </c>
+      <c r="E93" s="12" t="n"/>
+      <c r="F93" s="12" t="n"/>
+      <c r="G93" s="12" t="n"/>
       <c r="H93" s="12" t="n"/>
-      <c r="I93" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="J93" s="12" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I93" s="12" t="n"/>
+      <c r="J93" s="12" t="n"/>
       <c r="K93" s="13">
         <f>E93+F93+G93+H93+I93+J93</f>
         <v/>
@@ -10926,22 +10212,12 @@
         <f>IFERROR(VLOOKUP(C95,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E95" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F95" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G95" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E95" s="12" t="n"/>
+      <c r="F95" s="12" t="n"/>
+      <c r="G95" s="12" t="n"/>
       <c r="H95" s="12" t="n"/>
-      <c r="I95" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J95" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I95" s="12" t="n"/>
+      <c r="J95" s="12" t="n"/>
       <c r="K95" s="13">
         <f>E95+F95+G95+H95+I95+J95</f>
         <v/>
@@ -10993,22 +10269,12 @@
         <f>IFERROR(VLOOKUP(C96,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E96" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F96" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G96" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E96" s="12" t="n"/>
+      <c r="F96" s="12" t="n"/>
+      <c r="G96" s="12" t="n"/>
       <c r="H96" s="12" t="n"/>
-      <c r="I96" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J96" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I96" s="12" t="n"/>
+      <c r="J96" s="12" t="n"/>
       <c r="K96" s="13">
         <f>E96+F96+G96+H96+I96+J96</f>
         <v/>
@@ -11059,22 +10325,12 @@
         <f>IFERROR(VLOOKUP(C97,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E97" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F97" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G97" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E97" s="12" t="n"/>
+      <c r="F97" s="12" t="n"/>
+      <c r="G97" s="12" t="n"/>
       <c r="H97" s="12" t="n"/>
-      <c r="I97" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J97" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I97" s="12" t="n"/>
+      <c r="J97" s="12" t="n"/>
       <c r="K97" s="13">
         <f>E97+F97+G97+H97+I97+J97</f>
         <v/>
@@ -11125,22 +10381,12 @@
         <f>IFERROR(VLOOKUP(C98,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E98" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F98" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G98" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E98" s="12" t="n"/>
+      <c r="F98" s="12" t="n"/>
+      <c r="G98" s="12" t="n"/>
       <c r="H98" s="12" t="n"/>
-      <c r="I98" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J98" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I98" s="12" t="n"/>
+      <c r="J98" s="12" t="n"/>
       <c r="K98" s="13">
         <f>E98+F98+G98+H98+I98+J98</f>
         <v/>
@@ -11191,22 +10437,12 @@
         <f>IFERROR(VLOOKUP(C99,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E99" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F99" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G99" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E99" s="12" t="n"/>
+      <c r="F99" s="12" t="n"/>
+      <c r="G99" s="12" t="n"/>
       <c r="H99" s="12" t="n"/>
-      <c r="I99" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J99" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I99" s="12" t="n"/>
+      <c r="J99" s="12" t="n"/>
       <c r="K99" s="13">
         <f>E99+F99+G99+H99+I99+J99</f>
         <v/>
@@ -11257,22 +10493,12 @@
         <f>IFERROR(VLOOKUP(C100,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E100" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F100" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G100" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E100" s="12" t="n"/>
+      <c r="F100" s="12" t="n"/>
+      <c r="G100" s="12" t="n"/>
       <c r="H100" s="12" t="n"/>
-      <c r="I100" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J100" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I100" s="12" t="n"/>
+      <c r="J100" s="12" t="n"/>
       <c r="K100" s="13">
         <f>E100+F100+G100+H100+I100+J100</f>
         <v/>
@@ -11323,22 +10549,12 @@
         <f>IFERROR(VLOOKUP(C101,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E101" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F101" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G101" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E101" s="12" t="n"/>
+      <c r="F101" s="12" t="n"/>
+      <c r="G101" s="12" t="n"/>
       <c r="H101" s="12" t="n"/>
-      <c r="I101" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J101" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I101" s="12" t="n"/>
+      <c r="J101" s="12" t="n"/>
       <c r="K101" s="13">
         <f>E101+F101+G101+H101+I101+J101</f>
         <v/>
@@ -11389,22 +10605,12 @@
         <f>IFERROR(VLOOKUP(C102,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E102" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F102" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G102" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E102" s="12" t="n"/>
+      <c r="F102" s="12" t="n"/>
+      <c r="G102" s="12" t="n"/>
       <c r="H102" s="12" t="n"/>
-      <c r="I102" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J102" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I102" s="12" t="n"/>
+      <c r="J102" s="12" t="n"/>
       <c r="K102" s="13">
         <f>E102+F102+G102+H102+I102+J102</f>
         <v/>
@@ -11455,22 +10661,12 @@
         <f>IFERROR(VLOOKUP(C103,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E103" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F103" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G103" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E103" s="12" t="n"/>
+      <c r="F103" s="12" t="n"/>
+      <c r="G103" s="12" t="n"/>
       <c r="H103" s="12" t="n"/>
-      <c r="I103" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J103" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I103" s="12" t="n"/>
+      <c r="J103" s="12" t="n"/>
       <c r="K103" s="13">
         <f>E103+F103+G103+H103+I103+J103</f>
         <v/>
@@ -11521,22 +10717,12 @@
         <f>IFERROR(VLOOKUP(C104,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E104" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F104" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G104" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E104" s="12" t="n"/>
+      <c r="F104" s="12" t="n"/>
+      <c r="G104" s="12" t="n"/>
       <c r="H104" s="12" t="n"/>
-      <c r="I104" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J104" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I104" s="12" t="n"/>
+      <c r="J104" s="12" t="n"/>
       <c r="K104" s="13">
         <f>E104+F104+G104+H104+I104+J104</f>
         <v/>
@@ -11587,22 +10773,12 @@
         <f>IFERROR(VLOOKUP(C105,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E105" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F105" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G105" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E105" s="12" t="n"/>
+      <c r="F105" s="12" t="n"/>
+      <c r="G105" s="12" t="n"/>
       <c r="H105" s="12" t="n"/>
-      <c r="I105" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J105" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I105" s="12" t="n"/>
+      <c r="J105" s="12" t="n"/>
       <c r="K105" s="13">
         <f>E105+F105+G105+H105+I105+J105</f>
         <v/>
@@ -11653,22 +10829,12 @@
         <f>IFERROR(VLOOKUP(C106,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E106" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F106" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G106" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E106" s="12" t="n"/>
+      <c r="F106" s="12" t="n"/>
+      <c r="G106" s="12" t="n"/>
       <c r="H106" s="12" t="n"/>
-      <c r="I106" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J106" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I106" s="12" t="n"/>
+      <c r="J106" s="12" t="n"/>
       <c r="K106" s="13">
         <f>E106+F106+G106+H106+I106+J106</f>
         <v/>
@@ -11719,22 +10885,12 @@
         <f>IFERROR(VLOOKUP(C107,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E107" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F107" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G107" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E107" s="12" t="n"/>
+      <c r="F107" s="12" t="n"/>
+      <c r="G107" s="12" t="n"/>
       <c r="H107" s="12" t="n"/>
-      <c r="I107" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J107" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I107" s="12" t="n"/>
+      <c r="J107" s="12" t="n"/>
       <c r="K107" s="13">
         <f>E107+F107+G107+H107+I107+J107</f>
         <v/>
@@ -11785,22 +10941,12 @@
         <f>IFERROR(VLOOKUP(C108,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E108" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F108" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G108" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E108" s="12" t="n"/>
+      <c r="F108" s="12" t="n"/>
+      <c r="G108" s="12" t="n"/>
       <c r="H108" s="12" t="n"/>
-      <c r="I108" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J108" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I108" s="12" t="n"/>
+      <c r="J108" s="12" t="n"/>
       <c r="K108" s="13">
         <f>E108+F108+G108+H108+I108+J108</f>
         <v/>
@@ -11851,22 +10997,12 @@
         <f>IFERROR(VLOOKUP(C109,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E109" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F109" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G109" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E109" s="12" t="n"/>
+      <c r="F109" s="12" t="n"/>
+      <c r="G109" s="12" t="n"/>
       <c r="H109" s="12" t="n"/>
-      <c r="I109" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J109" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I109" s="12" t="n"/>
+      <c r="J109" s="12" t="n"/>
       <c r="K109" s="13">
         <f>E109+F109+G109+H109+I109+J109</f>
         <v/>
@@ -11917,22 +11053,12 @@
         <f>IFERROR(VLOOKUP(C110,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E110" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F110" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G110" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E110" s="12" t="n"/>
+      <c r="F110" s="12" t="n"/>
+      <c r="G110" s="12" t="n"/>
       <c r="H110" s="12" t="n"/>
-      <c r="I110" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J110" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I110" s="12" t="n"/>
+      <c r="J110" s="12" t="n"/>
       <c r="K110" s="13">
         <f>E110+F110+G110+H110+I110+J110</f>
         <v/>
@@ -11983,22 +11109,12 @@
         <f>IFERROR(VLOOKUP(C111,▼売上原票!$A:$P,8,0),0)</f>
         <v/>
       </c>
-      <c r="E111" s="12" t="n">
-        <v>120000</v>
-      </c>
-      <c r="F111" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="G111" s="12" t="n">
-        <v>18000</v>
-      </c>
+      <c r="E111" s="12" t="n"/>
+      <c r="F111" s="12" t="n"/>
+      <c r="G111" s="12" t="n"/>
       <c r="H111" s="12" t="n"/>
-      <c r="I111" s="12" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J111" s="12" t="n">
-        <v>12000</v>
-      </c>
+      <c r="I111" s="12" t="n"/>
+      <c r="J111" s="12" t="n"/>
       <c r="K111" s="13">
         <f>E111+F111+G111+H111+I111+J111</f>
         <v/>
@@ -12068,22 +11184,12 @@
         <f>IFERROR(VLOOKUP(C113,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E113" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F113" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G113" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E113" s="12" t="n"/>
+      <c r="F113" s="12" t="n"/>
+      <c r="G113" s="12" t="n"/>
       <c r="H113" s="12" t="n"/>
-      <c r="I113" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J113" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I113" s="12" t="n"/>
+      <c r="J113" s="12" t="n"/>
       <c r="K113" s="13">
         <f>E113+F113+G113+H113+I113+J113</f>
         <v/>
@@ -12135,22 +11241,12 @@
         <f>IFERROR(VLOOKUP(C114,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E114" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F114" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G114" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E114" s="12" t="n"/>
+      <c r="F114" s="12" t="n"/>
+      <c r="G114" s="12" t="n"/>
       <c r="H114" s="12" t="n"/>
-      <c r="I114" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J114" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I114" s="12" t="n"/>
+      <c r="J114" s="12" t="n"/>
       <c r="K114" s="13">
         <f>E114+F114+G114+H114+I114+J114</f>
         <v/>
@@ -12201,22 +11297,12 @@
         <f>IFERROR(VLOOKUP(C115,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E115" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F115" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G115" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E115" s="12" t="n"/>
+      <c r="F115" s="12" t="n"/>
+      <c r="G115" s="12" t="n"/>
       <c r="H115" s="12" t="n"/>
-      <c r="I115" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J115" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I115" s="12" t="n"/>
+      <c r="J115" s="12" t="n"/>
       <c r="K115" s="13">
         <f>E115+F115+G115+H115+I115+J115</f>
         <v/>
@@ -12267,22 +11353,12 @@
         <f>IFERROR(VLOOKUP(C116,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E116" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F116" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G116" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E116" s="12" t="n"/>
+      <c r="F116" s="12" t="n"/>
+      <c r="G116" s="12" t="n"/>
       <c r="H116" s="12" t="n"/>
-      <c r="I116" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J116" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I116" s="12" t="n"/>
+      <c r="J116" s="12" t="n"/>
       <c r="K116" s="13">
         <f>E116+F116+G116+H116+I116+J116</f>
         <v/>
@@ -12333,22 +11409,12 @@
         <f>IFERROR(VLOOKUP(C117,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E117" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F117" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G117" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E117" s="12" t="n"/>
+      <c r="F117" s="12" t="n"/>
+      <c r="G117" s="12" t="n"/>
       <c r="H117" s="12" t="n"/>
-      <c r="I117" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J117" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I117" s="12" t="n"/>
+      <c r="J117" s="12" t="n"/>
       <c r="K117" s="13">
         <f>E117+F117+G117+H117+I117+J117</f>
         <v/>
@@ -12399,22 +11465,12 @@
         <f>IFERROR(VLOOKUP(C118,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E118" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F118" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G118" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E118" s="12" t="n"/>
+      <c r="F118" s="12" t="n"/>
+      <c r="G118" s="12" t="n"/>
       <c r="H118" s="12" t="n"/>
-      <c r="I118" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J118" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I118" s="12" t="n"/>
+      <c r="J118" s="12" t="n"/>
       <c r="K118" s="13">
         <f>E118+F118+G118+H118+I118+J118</f>
         <v/>
@@ -12465,22 +11521,12 @@
         <f>IFERROR(VLOOKUP(C119,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E119" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F119" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G119" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E119" s="12" t="n"/>
+      <c r="F119" s="12" t="n"/>
+      <c r="G119" s="12" t="n"/>
       <c r="H119" s="12" t="n"/>
-      <c r="I119" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J119" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I119" s="12" t="n"/>
+      <c r="J119" s="12" t="n"/>
       <c r="K119" s="13">
         <f>E119+F119+G119+H119+I119+J119</f>
         <v/>
@@ -12531,22 +11577,12 @@
         <f>IFERROR(VLOOKUP(C120,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E120" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F120" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G120" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E120" s="12" t="n"/>
+      <c r="F120" s="12" t="n"/>
+      <c r="G120" s="12" t="n"/>
       <c r="H120" s="12" t="n"/>
-      <c r="I120" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J120" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I120" s="12" t="n"/>
+      <c r="J120" s="12" t="n"/>
       <c r="K120" s="13">
         <f>E120+F120+G120+H120+I120+J120</f>
         <v/>
@@ -12597,22 +11633,12 @@
         <f>IFERROR(VLOOKUP(C121,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E121" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F121" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G121" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E121" s="12" t="n"/>
+      <c r="F121" s="12" t="n"/>
+      <c r="G121" s="12" t="n"/>
       <c r="H121" s="12" t="n"/>
-      <c r="I121" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J121" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I121" s="12" t="n"/>
+      <c r="J121" s="12" t="n"/>
       <c r="K121" s="13">
         <f>E121+F121+G121+H121+I121+J121</f>
         <v/>
@@ -12663,22 +11689,12 @@
         <f>IFERROR(VLOOKUP(C122,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E122" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F122" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G122" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E122" s="12" t="n"/>
+      <c r="F122" s="12" t="n"/>
+      <c r="G122" s="12" t="n"/>
       <c r="H122" s="12" t="n"/>
-      <c r="I122" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J122" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I122" s="12" t="n"/>
+      <c r="J122" s="12" t="n"/>
       <c r="K122" s="13">
         <f>E122+F122+G122+H122+I122+J122</f>
         <v/>
@@ -12729,22 +11745,12 @@
         <f>IFERROR(VLOOKUP(C123,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E123" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F123" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G123" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E123" s="12" t="n"/>
+      <c r="F123" s="12" t="n"/>
+      <c r="G123" s="12" t="n"/>
       <c r="H123" s="12" t="n"/>
-      <c r="I123" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J123" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I123" s="12" t="n"/>
+      <c r="J123" s="12" t="n"/>
       <c r="K123" s="13">
         <f>E123+F123+G123+H123+I123+J123</f>
         <v/>
@@ -12795,22 +11801,12 @@
         <f>IFERROR(VLOOKUP(C124,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E124" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F124" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G124" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E124" s="12" t="n"/>
+      <c r="F124" s="12" t="n"/>
+      <c r="G124" s="12" t="n"/>
       <c r="H124" s="12" t="n"/>
-      <c r="I124" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J124" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I124" s="12" t="n"/>
+      <c r="J124" s="12" t="n"/>
       <c r="K124" s="13">
         <f>E124+F124+G124+H124+I124+J124</f>
         <v/>
@@ -12861,22 +11857,12 @@
         <f>IFERROR(VLOOKUP(C125,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E125" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F125" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G125" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E125" s="12" t="n"/>
+      <c r="F125" s="12" t="n"/>
+      <c r="G125" s="12" t="n"/>
       <c r="H125" s="12" t="n"/>
-      <c r="I125" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J125" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I125" s="12" t="n"/>
+      <c r="J125" s="12" t="n"/>
       <c r="K125" s="13">
         <f>E125+F125+G125+H125+I125+J125</f>
         <v/>
@@ -12927,22 +11913,12 @@
         <f>IFERROR(VLOOKUP(C126,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E126" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F126" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G126" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E126" s="12" t="n"/>
+      <c r="F126" s="12" t="n"/>
+      <c r="G126" s="12" t="n"/>
       <c r="H126" s="12" t="n"/>
-      <c r="I126" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J126" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I126" s="12" t="n"/>
+      <c r="J126" s="12" t="n"/>
       <c r="K126" s="13">
         <f>E126+F126+G126+H126+I126+J126</f>
         <v/>
@@ -12993,22 +11969,12 @@
         <f>IFERROR(VLOOKUP(C127,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E127" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F127" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G127" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E127" s="12" t="n"/>
+      <c r="F127" s="12" t="n"/>
+      <c r="G127" s="12" t="n"/>
       <c r="H127" s="12" t="n"/>
-      <c r="I127" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J127" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I127" s="12" t="n"/>
+      <c r="J127" s="12" t="n"/>
       <c r="K127" s="13">
         <f>E127+F127+G127+H127+I127+J127</f>
         <v/>
@@ -13059,22 +12025,12 @@
         <f>IFERROR(VLOOKUP(C128,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E128" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F128" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G128" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E128" s="12" t="n"/>
+      <c r="F128" s="12" t="n"/>
+      <c r="G128" s="12" t="n"/>
       <c r="H128" s="12" t="n"/>
-      <c r="I128" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J128" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I128" s="12" t="n"/>
+      <c r="J128" s="12" t="n"/>
       <c r="K128" s="13">
         <f>E128+F128+G128+H128+I128+J128</f>
         <v/>
@@ -13125,22 +12081,12 @@
         <f>IFERROR(VLOOKUP(C129,▼売上原票!$A:$P,9,0),0)</f>
         <v/>
       </c>
-      <c r="E129" s="12" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F129" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="G129" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E129" s="12" t="n"/>
+      <c r="F129" s="12" t="n"/>
+      <c r="G129" s="12" t="n"/>
       <c r="H129" s="12" t="n"/>
-      <c r="I129" s="12" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J129" s="12" t="n">
-        <v>3000</v>
-      </c>
+      <c r="I129" s="12" t="n"/>
+      <c r="J129" s="12" t="n"/>
       <c r="K129" s="13">
         <f>E129+F129+G129+H129+I129+J129</f>
         <v/>
@@ -13210,24 +12156,12 @@
         <f>IFERROR(VLOOKUP(C131,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E131" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F131" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G131" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H131" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I131" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J131" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E131" s="12" t="n"/>
+      <c r="F131" s="12" t="n"/>
+      <c r="G131" s="12" t="n"/>
+      <c r="H131" s="12" t="n"/>
+      <c r="I131" s="12" t="n"/>
+      <c r="J131" s="12" t="n"/>
       <c r="K131" s="13">
         <f>E131+F131+G131+H131+I131+J131</f>
         <v/>
@@ -13279,24 +12213,12 @@
         <f>IFERROR(VLOOKUP(C132,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E132" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F132" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G132" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H132" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I132" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J132" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E132" s="12" t="n"/>
+      <c r="F132" s="12" t="n"/>
+      <c r="G132" s="12" t="n"/>
+      <c r="H132" s="12" t="n"/>
+      <c r="I132" s="12" t="n"/>
+      <c r="J132" s="12" t="n"/>
       <c r="K132" s="13">
         <f>E132+F132+G132+H132+I132+J132</f>
         <v/>
@@ -13347,24 +12269,12 @@
         <f>IFERROR(VLOOKUP(C133,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E133" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F133" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G133" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H133" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I133" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J133" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E133" s="12" t="n"/>
+      <c r="F133" s="12" t="n"/>
+      <c r="G133" s="12" t="n"/>
+      <c r="H133" s="12" t="n"/>
+      <c r="I133" s="12" t="n"/>
+      <c r="J133" s="12" t="n"/>
       <c r="K133" s="13">
         <f>E133+F133+G133+H133+I133+J133</f>
         <v/>
@@ -13415,24 +12325,12 @@
         <f>IFERROR(VLOOKUP(C134,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E134" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F134" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G134" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H134" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I134" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J134" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E134" s="12" t="n"/>
+      <c r="F134" s="12" t="n"/>
+      <c r="G134" s="12" t="n"/>
+      <c r="H134" s="12" t="n"/>
+      <c r="I134" s="12" t="n"/>
+      <c r="J134" s="12" t="n"/>
       <c r="K134" s="13">
         <f>E134+F134+G134+H134+I134+J134</f>
         <v/>
@@ -13483,24 +12381,12 @@
         <f>IFERROR(VLOOKUP(C135,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E135" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F135" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G135" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H135" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I135" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J135" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E135" s="12" t="n"/>
+      <c r="F135" s="12" t="n"/>
+      <c r="G135" s="12" t="n"/>
+      <c r="H135" s="12" t="n"/>
+      <c r="I135" s="12" t="n"/>
+      <c r="J135" s="12" t="n"/>
       <c r="K135" s="13">
         <f>E135+F135+G135+H135+I135+J135</f>
         <v/>
@@ -13551,24 +12437,12 @@
         <f>IFERROR(VLOOKUP(C136,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E136" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F136" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G136" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H136" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I136" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J136" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E136" s="12" t="n"/>
+      <c r="F136" s="12" t="n"/>
+      <c r="G136" s="12" t="n"/>
+      <c r="H136" s="12" t="n"/>
+      <c r="I136" s="12" t="n"/>
+      <c r="J136" s="12" t="n"/>
       <c r="K136" s="13">
         <f>E136+F136+G136+H136+I136+J136</f>
         <v/>
@@ -13619,24 +12493,12 @@
         <f>IFERROR(VLOOKUP(C137,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E137" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F137" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G137" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H137" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I137" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J137" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E137" s="12" t="n"/>
+      <c r="F137" s="12" t="n"/>
+      <c r="G137" s="12" t="n"/>
+      <c r="H137" s="12" t="n"/>
+      <c r="I137" s="12" t="n"/>
+      <c r="J137" s="12" t="n"/>
       <c r="K137" s="13">
         <f>E137+F137+G137+H137+I137+J137</f>
         <v/>
@@ -13687,24 +12549,12 @@
         <f>IFERROR(VLOOKUP(C138,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E138" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F138" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G138" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H138" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I138" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J138" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E138" s="12" t="n"/>
+      <c r="F138" s="12" t="n"/>
+      <c r="G138" s="12" t="n"/>
+      <c r="H138" s="12" t="n"/>
+      <c r="I138" s="12" t="n"/>
+      <c r="J138" s="12" t="n"/>
       <c r="K138" s="13">
         <f>E138+F138+G138+H138+I138+J138</f>
         <v/>
@@ -13755,24 +12605,12 @@
         <f>IFERROR(VLOOKUP(C139,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E139" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F139" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G139" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H139" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I139" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J139" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E139" s="12" t="n"/>
+      <c r="F139" s="12" t="n"/>
+      <c r="G139" s="12" t="n"/>
+      <c r="H139" s="12" t="n"/>
+      <c r="I139" s="12" t="n"/>
+      <c r="J139" s="12" t="n"/>
       <c r="K139" s="13">
         <f>E139+F139+G139+H139+I139+J139</f>
         <v/>
@@ -13823,24 +12661,12 @@
         <f>IFERROR(VLOOKUP(C140,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E140" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F140" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G140" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H140" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I140" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J140" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E140" s="12" t="n"/>
+      <c r="F140" s="12" t="n"/>
+      <c r="G140" s="12" t="n"/>
+      <c r="H140" s="12" t="n"/>
+      <c r="I140" s="12" t="n"/>
+      <c r="J140" s="12" t="n"/>
       <c r="K140" s="13">
         <f>E140+F140+G140+H140+I140+J140</f>
         <v/>
@@ -13891,24 +12717,12 @@
         <f>IFERROR(VLOOKUP(C141,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E141" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F141" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G141" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H141" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I141" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J141" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E141" s="12" t="n"/>
+      <c r="F141" s="12" t="n"/>
+      <c r="G141" s="12" t="n"/>
+      <c r="H141" s="12" t="n"/>
+      <c r="I141" s="12" t="n"/>
+      <c r="J141" s="12" t="n"/>
       <c r="K141" s="13">
         <f>E141+F141+G141+H141+I141+J141</f>
         <v/>
@@ -13959,24 +12773,12 @@
         <f>IFERROR(VLOOKUP(C142,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E142" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F142" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G142" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H142" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I142" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J142" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E142" s="12" t="n"/>
+      <c r="F142" s="12" t="n"/>
+      <c r="G142" s="12" t="n"/>
+      <c r="H142" s="12" t="n"/>
+      <c r="I142" s="12" t="n"/>
+      <c r="J142" s="12" t="n"/>
       <c r="K142" s="13">
         <f>E142+F142+G142+H142+I142+J142</f>
         <v/>
@@ -14027,24 +12829,12 @@
         <f>IFERROR(VLOOKUP(C143,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E143" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F143" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G143" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H143" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I143" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J143" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E143" s="12" t="n"/>
+      <c r="F143" s="12" t="n"/>
+      <c r="G143" s="12" t="n"/>
+      <c r="H143" s="12" t="n"/>
+      <c r="I143" s="12" t="n"/>
+      <c r="J143" s="12" t="n"/>
       <c r="K143" s="13">
         <f>E143+F143+G143+H143+I143+J143</f>
         <v/>
@@ -14095,24 +12885,12 @@
         <f>IFERROR(VLOOKUP(C144,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E144" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F144" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G144" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H144" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I144" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J144" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E144" s="12" t="n"/>
+      <c r="F144" s="12" t="n"/>
+      <c r="G144" s="12" t="n"/>
+      <c r="H144" s="12" t="n"/>
+      <c r="I144" s="12" t="n"/>
+      <c r="J144" s="12" t="n"/>
       <c r="K144" s="13">
         <f>E144+F144+G144+H144+I144+J144</f>
         <v/>
@@ -14163,24 +12941,12 @@
         <f>IFERROR(VLOOKUP(C145,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E145" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F145" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G145" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H145" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I145" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J145" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E145" s="12" t="n"/>
+      <c r="F145" s="12" t="n"/>
+      <c r="G145" s="12" t="n"/>
+      <c r="H145" s="12" t="n"/>
+      <c r="I145" s="12" t="n"/>
+      <c r="J145" s="12" t="n"/>
       <c r="K145" s="13">
         <f>E145+F145+G145+H145+I145+J145</f>
         <v/>
@@ -14231,24 +12997,12 @@
         <f>IFERROR(VLOOKUP(C146,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E146" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F146" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G146" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H146" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I146" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J146" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E146" s="12" t="n"/>
+      <c r="F146" s="12" t="n"/>
+      <c r="G146" s="12" t="n"/>
+      <c r="H146" s="12" t="n"/>
+      <c r="I146" s="12" t="n"/>
+      <c r="J146" s="12" t="n"/>
       <c r="K146" s="13">
         <f>E146+F146+G146+H146+I146+J146</f>
         <v/>
@@ -14299,24 +13053,12 @@
         <f>IFERROR(VLOOKUP(C147,▼売上原票!$A:$P,10,0),0)</f>
         <v/>
       </c>
-      <c r="E147" s="12" t="n">
-        <v>850000</v>
-      </c>
-      <c r="F147" s="12" t="n">
-        <v>248000</v>
-      </c>
-      <c r="G147" s="12" t="n">
-        <v>118000</v>
-      </c>
-      <c r="H147" s="12" t="n">
-        <v>580000</v>
-      </c>
-      <c r="I147" s="12" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J147" s="12" t="n">
-        <v>62000</v>
-      </c>
+      <c r="E147" s="12" t="n"/>
+      <c r="F147" s="12" t="n"/>
+      <c r="G147" s="12" t="n"/>
+      <c r="H147" s="12" t="n"/>
+      <c r="I147" s="12" t="n"/>
+      <c r="J147" s="12" t="n"/>
       <c r="K147" s="13">
         <f>E147+F147+G147+H147+I147+J147</f>
         <v/>
@@ -14386,24 +13128,12 @@
         <f>IFERROR(VLOOKUP(C149,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E149" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F149" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G149" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H149" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I149" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J149" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E149" s="12" t="n"/>
+      <c r="F149" s="12" t="n"/>
+      <c r="G149" s="12" t="n"/>
+      <c r="H149" s="12" t="n"/>
+      <c r="I149" s="12" t="n"/>
+      <c r="J149" s="12" t="n"/>
       <c r="K149" s="13">
         <f>E149+F149+G149+H149+I149+J149</f>
         <v/>
@@ -14455,24 +13185,12 @@
         <f>IFERROR(VLOOKUP(C150,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E150" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F150" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G150" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H150" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I150" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J150" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E150" s="12" t="n"/>
+      <c r="F150" s="12" t="n"/>
+      <c r="G150" s="12" t="n"/>
+      <c r="H150" s="12" t="n"/>
+      <c r="I150" s="12" t="n"/>
+      <c r="J150" s="12" t="n"/>
       <c r="K150" s="13">
         <f>E150+F150+G150+H150+I150+J150</f>
         <v/>
@@ -14523,24 +13241,12 @@
         <f>IFERROR(VLOOKUP(C151,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E151" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F151" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G151" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H151" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I151" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J151" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E151" s="12" t="n"/>
+      <c r="F151" s="12" t="n"/>
+      <c r="G151" s="12" t="n"/>
+      <c r="H151" s="12" t="n"/>
+      <c r="I151" s="12" t="n"/>
+      <c r="J151" s="12" t="n"/>
       <c r="K151" s="13">
         <f>E151+F151+G151+H151+I151+J151</f>
         <v/>
@@ -14591,24 +13297,12 @@
         <f>IFERROR(VLOOKUP(C152,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E152" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F152" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G152" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H152" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I152" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J152" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E152" s="12" t="n"/>
+      <c r="F152" s="12" t="n"/>
+      <c r="G152" s="12" t="n"/>
+      <c r="H152" s="12" t="n"/>
+      <c r="I152" s="12" t="n"/>
+      <c r="J152" s="12" t="n"/>
       <c r="K152" s="13">
         <f>E152+F152+G152+H152+I152+J152</f>
         <v/>
@@ -14659,24 +13353,12 @@
         <f>IFERROR(VLOOKUP(C153,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E153" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F153" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G153" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H153" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I153" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J153" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E153" s="12" t="n"/>
+      <c r="F153" s="12" t="n"/>
+      <c r="G153" s="12" t="n"/>
+      <c r="H153" s="12" t="n"/>
+      <c r="I153" s="12" t="n"/>
+      <c r="J153" s="12" t="n"/>
       <c r="K153" s="13">
         <f>E153+F153+G153+H153+I153+J153</f>
         <v/>
@@ -14727,24 +13409,12 @@
         <f>IFERROR(VLOOKUP(C154,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E154" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F154" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G154" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H154" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I154" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J154" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E154" s="12" t="n"/>
+      <c r="F154" s="12" t="n"/>
+      <c r="G154" s="12" t="n"/>
+      <c r="H154" s="12" t="n"/>
+      <c r="I154" s="12" t="n"/>
+      <c r="J154" s="12" t="n"/>
       <c r="K154" s="13">
         <f>E154+F154+G154+H154+I154+J154</f>
         <v/>
@@ -14795,24 +13465,12 @@
         <f>IFERROR(VLOOKUP(C155,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E155" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F155" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G155" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H155" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I155" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J155" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E155" s="12" t="n"/>
+      <c r="F155" s="12" t="n"/>
+      <c r="G155" s="12" t="n"/>
+      <c r="H155" s="12" t="n"/>
+      <c r="I155" s="12" t="n"/>
+      <c r="J155" s="12" t="n"/>
       <c r="K155" s="13">
         <f>E155+F155+G155+H155+I155+J155</f>
         <v/>
@@ -14863,24 +13521,12 @@
         <f>IFERROR(VLOOKUP(C156,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E156" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F156" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G156" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H156" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I156" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J156" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E156" s="12" t="n"/>
+      <c r="F156" s="12" t="n"/>
+      <c r="G156" s="12" t="n"/>
+      <c r="H156" s="12" t="n"/>
+      <c r="I156" s="12" t="n"/>
+      <c r="J156" s="12" t="n"/>
       <c r="K156" s="13">
         <f>E156+F156+G156+H156+I156+J156</f>
         <v/>
@@ -14931,24 +13577,12 @@
         <f>IFERROR(VLOOKUP(C157,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E157" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F157" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G157" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H157" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I157" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J157" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E157" s="12" t="n"/>
+      <c r="F157" s="12" t="n"/>
+      <c r="G157" s="12" t="n"/>
+      <c r="H157" s="12" t="n"/>
+      <c r="I157" s="12" t="n"/>
+      <c r="J157" s="12" t="n"/>
       <c r="K157" s="13">
         <f>E157+F157+G157+H157+I157+J157</f>
         <v/>
@@ -14999,24 +13633,12 @@
         <f>IFERROR(VLOOKUP(C158,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E158" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F158" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G158" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H158" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I158" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J158" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E158" s="12" t="n"/>
+      <c r="F158" s="12" t="n"/>
+      <c r="G158" s="12" t="n"/>
+      <c r="H158" s="12" t="n"/>
+      <c r="I158" s="12" t="n"/>
+      <c r="J158" s="12" t="n"/>
       <c r="K158" s="13">
         <f>E158+F158+G158+H158+I158+J158</f>
         <v/>
@@ -15067,24 +13689,12 @@
         <f>IFERROR(VLOOKUP(C159,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E159" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F159" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G159" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H159" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I159" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J159" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E159" s="12" t="n"/>
+      <c r="F159" s="12" t="n"/>
+      <c r="G159" s="12" t="n"/>
+      <c r="H159" s="12" t="n"/>
+      <c r="I159" s="12" t="n"/>
+      <c r="J159" s="12" t="n"/>
       <c r="K159" s="13">
         <f>E159+F159+G159+H159+I159+J159</f>
         <v/>
@@ -15135,24 +13745,12 @@
         <f>IFERROR(VLOOKUP(C160,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E160" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F160" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G160" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H160" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I160" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J160" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E160" s="12" t="n"/>
+      <c r="F160" s="12" t="n"/>
+      <c r="G160" s="12" t="n"/>
+      <c r="H160" s="12" t="n"/>
+      <c r="I160" s="12" t="n"/>
+      <c r="J160" s="12" t="n"/>
       <c r="K160" s="13">
         <f>E160+F160+G160+H160+I160+J160</f>
         <v/>
@@ -15203,24 +13801,12 @@
         <f>IFERROR(VLOOKUP(C161,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E161" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F161" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G161" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H161" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I161" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J161" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E161" s="12" t="n"/>
+      <c r="F161" s="12" t="n"/>
+      <c r="G161" s="12" t="n"/>
+      <c r="H161" s="12" t="n"/>
+      <c r="I161" s="12" t="n"/>
+      <c r="J161" s="12" t="n"/>
       <c r="K161" s="13">
         <f>E161+F161+G161+H161+I161+J161</f>
         <v/>
@@ -15271,24 +13857,12 @@
         <f>IFERROR(VLOOKUP(C162,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E162" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F162" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G162" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H162" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I162" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J162" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E162" s="12" t="n"/>
+      <c r="F162" s="12" t="n"/>
+      <c r="G162" s="12" t="n"/>
+      <c r="H162" s="12" t="n"/>
+      <c r="I162" s="12" t="n"/>
+      <c r="J162" s="12" t="n"/>
       <c r="K162" s="13">
         <f>E162+F162+G162+H162+I162+J162</f>
         <v/>
@@ -15339,24 +13913,12 @@
         <f>IFERROR(VLOOKUP(C163,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E163" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F163" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G163" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H163" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I163" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J163" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E163" s="12" t="n"/>
+      <c r="F163" s="12" t="n"/>
+      <c r="G163" s="12" t="n"/>
+      <c r="H163" s="12" t="n"/>
+      <c r="I163" s="12" t="n"/>
+      <c r="J163" s="12" t="n"/>
       <c r="K163" s="13">
         <f>E163+F163+G163+H163+I163+J163</f>
         <v/>
@@ -15407,24 +13969,12 @@
         <f>IFERROR(VLOOKUP(C164,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E164" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F164" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G164" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H164" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I164" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J164" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E164" s="12" t="n"/>
+      <c r="F164" s="12" t="n"/>
+      <c r="G164" s="12" t="n"/>
+      <c r="H164" s="12" t="n"/>
+      <c r="I164" s="12" t="n"/>
+      <c r="J164" s="12" t="n"/>
       <c r="K164" s="13">
         <f>E164+F164+G164+H164+I164+J164</f>
         <v/>
@@ -15475,24 +14025,12 @@
         <f>IFERROR(VLOOKUP(C165,▼売上原票!$A:$P,11,0),0)</f>
         <v/>
       </c>
-      <c r="E165" s="12" t="n">
-        <v>280000</v>
-      </c>
-      <c r="F165" s="12" t="n">
-        <v>82000</v>
-      </c>
-      <c r="G165" s="12" t="n">
-        <v>38000</v>
-      </c>
-      <c r="H165" s="12" t="n">
-        <v>195000</v>
-      </c>
-      <c r="I165" s="12" t="n">
-        <v>32000</v>
-      </c>
-      <c r="J165" s="12" t="n">
-        <v>20000</v>
-      </c>
+      <c r="E165" s="12" t="n"/>
+      <c r="F165" s="12" t="n"/>
+      <c r="G165" s="12" t="n"/>
+      <c r="H165" s="12" t="n"/>
+      <c r="I165" s="12" t="n"/>
+      <c r="J165" s="12" t="n"/>
       <c r="K165" s="13">
         <f>E165+F165+G165+H165+I165+J165</f>
         <v/>
@@ -15562,22 +14100,12 @@
         <f>IFERROR(VLOOKUP(C167,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E167" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F167" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G167" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E167" s="12" t="n"/>
+      <c r="F167" s="12" t="n"/>
+      <c r="G167" s="12" t="n"/>
       <c r="H167" s="12" t="n"/>
-      <c r="I167" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J167" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I167" s="12" t="n"/>
+      <c r="J167" s="12" t="n"/>
       <c r="K167" s="13">
         <f>E167+F167+G167+H167+I167+J167</f>
         <v/>
@@ -15629,22 +14157,12 @@
         <f>IFERROR(VLOOKUP(C168,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E168" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F168" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G168" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E168" s="12" t="n"/>
+      <c r="F168" s="12" t="n"/>
+      <c r="G168" s="12" t="n"/>
       <c r="H168" s="12" t="n"/>
-      <c r="I168" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J168" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I168" s="12" t="n"/>
+      <c r="J168" s="12" t="n"/>
       <c r="K168" s="13">
         <f>E168+F168+G168+H168+I168+J168</f>
         <v/>
@@ -15695,22 +14213,12 @@
         <f>IFERROR(VLOOKUP(C169,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E169" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F169" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G169" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E169" s="12" t="n"/>
+      <c r="F169" s="12" t="n"/>
+      <c r="G169" s="12" t="n"/>
       <c r="H169" s="12" t="n"/>
-      <c r="I169" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J169" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I169" s="12" t="n"/>
+      <c r="J169" s="12" t="n"/>
       <c r="K169" s="13">
         <f>E169+F169+G169+H169+I169+J169</f>
         <v/>
@@ -15761,22 +14269,12 @@
         <f>IFERROR(VLOOKUP(C170,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E170" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F170" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G170" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E170" s="12" t="n"/>
+      <c r="F170" s="12" t="n"/>
+      <c r="G170" s="12" t="n"/>
       <c r="H170" s="12" t="n"/>
-      <c r="I170" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J170" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I170" s="12" t="n"/>
+      <c r="J170" s="12" t="n"/>
       <c r="K170" s="13">
         <f>E170+F170+G170+H170+I170+J170</f>
         <v/>
@@ -15827,22 +14325,12 @@
         <f>IFERROR(VLOOKUP(C171,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E171" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F171" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G171" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E171" s="12" t="n"/>
+      <c r="F171" s="12" t="n"/>
+      <c r="G171" s="12" t="n"/>
       <c r="H171" s="12" t="n"/>
-      <c r="I171" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J171" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I171" s="12" t="n"/>
+      <c r="J171" s="12" t="n"/>
       <c r="K171" s="13">
         <f>E171+F171+G171+H171+I171+J171</f>
         <v/>
@@ -15893,22 +14381,12 @@
         <f>IFERROR(VLOOKUP(C172,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E172" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F172" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G172" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E172" s="12" t="n"/>
+      <c r="F172" s="12" t="n"/>
+      <c r="G172" s="12" t="n"/>
       <c r="H172" s="12" t="n"/>
-      <c r="I172" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J172" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I172" s="12" t="n"/>
+      <c r="J172" s="12" t="n"/>
       <c r="K172" s="13">
         <f>E172+F172+G172+H172+I172+J172</f>
         <v/>
@@ -15959,22 +14437,12 @@
         <f>IFERROR(VLOOKUP(C173,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E173" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F173" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G173" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E173" s="12" t="n"/>
+      <c r="F173" s="12" t="n"/>
+      <c r="G173" s="12" t="n"/>
       <c r="H173" s="12" t="n"/>
-      <c r="I173" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J173" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I173" s="12" t="n"/>
+      <c r="J173" s="12" t="n"/>
       <c r="K173" s="13">
         <f>E173+F173+G173+H173+I173+J173</f>
         <v/>
@@ -16025,22 +14493,12 @@
         <f>IFERROR(VLOOKUP(C174,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E174" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F174" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G174" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E174" s="12" t="n"/>
+      <c r="F174" s="12" t="n"/>
+      <c r="G174" s="12" t="n"/>
       <c r="H174" s="12" t="n"/>
-      <c r="I174" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J174" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I174" s="12" t="n"/>
+      <c r="J174" s="12" t="n"/>
       <c r="K174" s="13">
         <f>E174+F174+G174+H174+I174+J174</f>
         <v/>
@@ -16091,22 +14549,12 @@
         <f>IFERROR(VLOOKUP(C175,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E175" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F175" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G175" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E175" s="12" t="n"/>
+      <c r="F175" s="12" t="n"/>
+      <c r="G175" s="12" t="n"/>
       <c r="H175" s="12" t="n"/>
-      <c r="I175" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J175" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I175" s="12" t="n"/>
+      <c r="J175" s="12" t="n"/>
       <c r="K175" s="13">
         <f>E175+F175+G175+H175+I175+J175</f>
         <v/>
@@ -16157,22 +14605,12 @@
         <f>IFERROR(VLOOKUP(C176,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E176" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F176" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G176" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E176" s="12" t="n"/>
+      <c r="F176" s="12" t="n"/>
+      <c r="G176" s="12" t="n"/>
       <c r="H176" s="12" t="n"/>
-      <c r="I176" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J176" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I176" s="12" t="n"/>
+      <c r="J176" s="12" t="n"/>
       <c r="K176" s="13">
         <f>E176+F176+G176+H176+I176+J176</f>
         <v/>
@@ -16223,22 +14661,12 @@
         <f>IFERROR(VLOOKUP(C177,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E177" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F177" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G177" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E177" s="12" t="n"/>
+      <c r="F177" s="12" t="n"/>
+      <c r="G177" s="12" t="n"/>
       <c r="H177" s="12" t="n"/>
-      <c r="I177" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J177" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I177" s="12" t="n"/>
+      <c r="J177" s="12" t="n"/>
       <c r="K177" s="13">
         <f>E177+F177+G177+H177+I177+J177</f>
         <v/>
@@ -16289,22 +14717,12 @@
         <f>IFERROR(VLOOKUP(C178,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E178" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F178" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G178" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E178" s="12" t="n"/>
+      <c r="F178" s="12" t="n"/>
+      <c r="G178" s="12" t="n"/>
       <c r="H178" s="12" t="n"/>
-      <c r="I178" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J178" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I178" s="12" t="n"/>
+      <c r="J178" s="12" t="n"/>
       <c r="K178" s="13">
         <f>E178+F178+G178+H178+I178+J178</f>
         <v/>
@@ -16355,22 +14773,12 @@
         <f>IFERROR(VLOOKUP(C179,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E179" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F179" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G179" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E179" s="12" t="n"/>
+      <c r="F179" s="12" t="n"/>
+      <c r="G179" s="12" t="n"/>
       <c r="H179" s="12" t="n"/>
-      <c r="I179" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J179" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I179" s="12" t="n"/>
+      <c r="J179" s="12" t="n"/>
       <c r="K179" s="13">
         <f>E179+F179+G179+H179+I179+J179</f>
         <v/>
@@ -16421,22 +14829,12 @@
         <f>IFERROR(VLOOKUP(C180,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E180" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F180" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G180" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E180" s="12" t="n"/>
+      <c r="F180" s="12" t="n"/>
+      <c r="G180" s="12" t="n"/>
       <c r="H180" s="12" t="n"/>
-      <c r="I180" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J180" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I180" s="12" t="n"/>
+      <c r="J180" s="12" t="n"/>
       <c r="K180" s="13">
         <f>E180+F180+G180+H180+I180+J180</f>
         <v/>
@@ -16487,22 +14885,12 @@
         <f>IFERROR(VLOOKUP(C181,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E181" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F181" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G181" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E181" s="12" t="n"/>
+      <c r="F181" s="12" t="n"/>
+      <c r="G181" s="12" t="n"/>
       <c r="H181" s="12" t="n"/>
-      <c r="I181" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J181" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I181" s="12" t="n"/>
+      <c r="J181" s="12" t="n"/>
       <c r="K181" s="13">
         <f>E181+F181+G181+H181+I181+J181</f>
         <v/>
@@ -16553,22 +14941,12 @@
         <f>IFERROR(VLOOKUP(C182,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E182" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F182" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G182" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E182" s="12" t="n"/>
+      <c r="F182" s="12" t="n"/>
+      <c r="G182" s="12" t="n"/>
       <c r="H182" s="12" t="n"/>
-      <c r="I182" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J182" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I182" s="12" t="n"/>
+      <c r="J182" s="12" t="n"/>
       <c r="K182" s="13">
         <f>E182+F182+G182+H182+I182+J182</f>
         <v/>
@@ -16619,22 +14997,12 @@
         <f>IFERROR(VLOOKUP(C183,▼売上原票!$A:$P,12,0),0)</f>
         <v/>
       </c>
-      <c r="E183" s="12" t="n">
-        <v>15000</v>
-      </c>
-      <c r="F183" s="12" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G183" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="E183" s="12" t="n"/>
+      <c r="F183" s="12" t="n"/>
+      <c r="G183" s="12" t="n"/>
       <c r="H183" s="12" t="n"/>
-      <c r="I183" s="12" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J183" s="12" t="n">
-        <v>2000</v>
-      </c>
+      <c r="I183" s="12" t="n"/>
+      <c r="J183" s="12" t="n"/>
       <c r="K183" s="13">
         <f>E183+F183+G183+H183+I183+J183</f>
         <v/>
@@ -16704,22 +15072,12 @@
         <f>IFERROR(VLOOKUP(C185,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E185" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F185" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G185" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E185" s="12" t="n"/>
+      <c r="F185" s="12" t="n"/>
+      <c r="G185" s="12" t="n"/>
       <c r="H185" s="12" t="n"/>
-      <c r="I185" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J185" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I185" s="12" t="n"/>
+      <c r="J185" s="12" t="n"/>
       <c r="K185" s="13">
         <f>E185+F185+G185+H185+I185+J185</f>
         <v/>
@@ -16771,22 +15129,12 @@
         <f>IFERROR(VLOOKUP(C186,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E186" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F186" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G186" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E186" s="12" t="n"/>
+      <c r="F186" s="12" t="n"/>
+      <c r="G186" s="12" t="n"/>
       <c r="H186" s="12" t="n"/>
-      <c r="I186" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J186" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I186" s="12" t="n"/>
+      <c r="J186" s="12" t="n"/>
       <c r="K186" s="13">
         <f>E186+F186+G186+H186+I186+J186</f>
         <v/>
@@ -16837,22 +15185,12 @@
         <f>IFERROR(VLOOKUP(C187,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E187" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F187" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G187" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E187" s="12" t="n"/>
+      <c r="F187" s="12" t="n"/>
+      <c r="G187" s="12" t="n"/>
       <c r="H187" s="12" t="n"/>
-      <c r="I187" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J187" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I187" s="12" t="n"/>
+      <c r="J187" s="12" t="n"/>
       <c r="K187" s="13">
         <f>E187+F187+G187+H187+I187+J187</f>
         <v/>
@@ -16903,22 +15241,12 @@
         <f>IFERROR(VLOOKUP(C188,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E188" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F188" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G188" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E188" s="12" t="n"/>
+      <c r="F188" s="12" t="n"/>
+      <c r="G188" s="12" t="n"/>
       <c r="H188" s="12" t="n"/>
-      <c r="I188" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J188" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I188" s="12" t="n"/>
+      <c r="J188" s="12" t="n"/>
       <c r="K188" s="13">
         <f>E188+F188+G188+H188+I188+J188</f>
         <v/>
@@ -16969,22 +15297,12 @@
         <f>IFERROR(VLOOKUP(C189,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E189" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F189" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G189" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E189" s="12" t="n"/>
+      <c r="F189" s="12" t="n"/>
+      <c r="G189" s="12" t="n"/>
       <c r="H189" s="12" t="n"/>
-      <c r="I189" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J189" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I189" s="12" t="n"/>
+      <c r="J189" s="12" t="n"/>
       <c r="K189" s="13">
         <f>E189+F189+G189+H189+I189+J189</f>
         <v/>
@@ -17035,22 +15353,12 @@
         <f>IFERROR(VLOOKUP(C190,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E190" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F190" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G190" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E190" s="12" t="n"/>
+      <c r="F190" s="12" t="n"/>
+      <c r="G190" s="12" t="n"/>
       <c r="H190" s="12" t="n"/>
-      <c r="I190" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J190" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I190" s="12" t="n"/>
+      <c r="J190" s="12" t="n"/>
       <c r="K190" s="13">
         <f>E190+F190+G190+H190+I190+J190</f>
         <v/>
@@ -17101,22 +15409,12 @@
         <f>IFERROR(VLOOKUP(C191,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E191" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F191" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G191" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E191" s="12" t="n"/>
+      <c r="F191" s="12" t="n"/>
+      <c r="G191" s="12" t="n"/>
       <c r="H191" s="12" t="n"/>
-      <c r="I191" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J191" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I191" s="12" t="n"/>
+      <c r="J191" s="12" t="n"/>
       <c r="K191" s="13">
         <f>E191+F191+G191+H191+I191+J191</f>
         <v/>
@@ -17167,22 +15465,12 @@
         <f>IFERROR(VLOOKUP(C192,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E192" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F192" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G192" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E192" s="12" t="n"/>
+      <c r="F192" s="12" t="n"/>
+      <c r="G192" s="12" t="n"/>
       <c r="H192" s="12" t="n"/>
-      <c r="I192" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J192" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I192" s="12" t="n"/>
+      <c r="J192" s="12" t="n"/>
       <c r="K192" s="13">
         <f>E192+F192+G192+H192+I192+J192</f>
         <v/>
@@ -17233,22 +15521,12 @@
         <f>IFERROR(VLOOKUP(C193,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E193" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F193" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G193" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E193" s="12" t="n"/>
+      <c r="F193" s="12" t="n"/>
+      <c r="G193" s="12" t="n"/>
       <c r="H193" s="12" t="n"/>
-      <c r="I193" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J193" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I193" s="12" t="n"/>
+      <c r="J193" s="12" t="n"/>
       <c r="K193" s="13">
         <f>E193+F193+G193+H193+I193+J193</f>
         <v/>
@@ -17299,22 +15577,12 @@
         <f>IFERROR(VLOOKUP(C194,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E194" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F194" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G194" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E194" s="12" t="n"/>
+      <c r="F194" s="12" t="n"/>
+      <c r="G194" s="12" t="n"/>
       <c r="H194" s="12" t="n"/>
-      <c r="I194" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J194" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I194" s="12" t="n"/>
+      <c r="J194" s="12" t="n"/>
       <c r="K194" s="13">
         <f>E194+F194+G194+H194+I194+J194</f>
         <v/>
@@ -17365,22 +15633,12 @@
         <f>IFERROR(VLOOKUP(C195,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E195" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F195" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G195" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E195" s="12" t="n"/>
+      <c r="F195" s="12" t="n"/>
+      <c r="G195" s="12" t="n"/>
       <c r="H195" s="12" t="n"/>
-      <c r="I195" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J195" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I195" s="12" t="n"/>
+      <c r="J195" s="12" t="n"/>
       <c r="K195" s="13">
         <f>E195+F195+G195+H195+I195+J195</f>
         <v/>
@@ -17431,22 +15689,12 @@
         <f>IFERROR(VLOOKUP(C196,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E196" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F196" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G196" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E196" s="12" t="n"/>
+      <c r="F196" s="12" t="n"/>
+      <c r="G196" s="12" t="n"/>
       <c r="H196" s="12" t="n"/>
-      <c r="I196" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J196" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I196" s="12" t="n"/>
+      <c r="J196" s="12" t="n"/>
       <c r="K196" s="13">
         <f>E196+F196+G196+H196+I196+J196</f>
         <v/>
@@ -17497,22 +15745,12 @@
         <f>IFERROR(VLOOKUP(C197,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E197" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F197" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G197" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E197" s="12" t="n"/>
+      <c r="F197" s="12" t="n"/>
+      <c r="G197" s="12" t="n"/>
       <c r="H197" s="12" t="n"/>
-      <c r="I197" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J197" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I197" s="12" t="n"/>
+      <c r="J197" s="12" t="n"/>
       <c r="K197" s="13">
         <f>E197+F197+G197+H197+I197+J197</f>
         <v/>
@@ -17563,22 +15801,12 @@
         <f>IFERROR(VLOOKUP(C198,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E198" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F198" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G198" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E198" s="12" t="n"/>
+      <c r="F198" s="12" t="n"/>
+      <c r="G198" s="12" t="n"/>
       <c r="H198" s="12" t="n"/>
-      <c r="I198" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J198" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I198" s="12" t="n"/>
+      <c r="J198" s="12" t="n"/>
       <c r="K198" s="13">
         <f>E198+F198+G198+H198+I198+J198</f>
         <v/>
@@ -17629,22 +15857,12 @@
         <f>IFERROR(VLOOKUP(C199,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E199" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F199" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G199" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E199" s="12" t="n"/>
+      <c r="F199" s="12" t="n"/>
+      <c r="G199" s="12" t="n"/>
       <c r="H199" s="12" t="n"/>
-      <c r="I199" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J199" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I199" s="12" t="n"/>
+      <c r="J199" s="12" t="n"/>
       <c r="K199" s="13">
         <f>E199+F199+G199+H199+I199+J199</f>
         <v/>
@@ -17695,22 +15913,12 @@
         <f>IFERROR(VLOOKUP(C200,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E200" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F200" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G200" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E200" s="12" t="n"/>
+      <c r="F200" s="12" t="n"/>
+      <c r="G200" s="12" t="n"/>
       <c r="H200" s="12" t="n"/>
-      <c r="I200" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J200" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I200" s="12" t="n"/>
+      <c r="J200" s="12" t="n"/>
       <c r="K200" s="13">
         <f>E200+F200+G200+H200+I200+J200</f>
         <v/>
@@ -17761,22 +15969,12 @@
         <f>IFERROR(VLOOKUP(C201,▼売上原票!$A:$P,13,0),0)</f>
         <v/>
       </c>
-      <c r="E201" s="12" t="n">
-        <v>35000</v>
-      </c>
-      <c r="F201" s="12" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G201" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="E201" s="12" t="n"/>
+      <c r="F201" s="12" t="n"/>
+      <c r="G201" s="12" t="n"/>
       <c r="H201" s="12" t="n"/>
-      <c r="I201" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J201" s="12" t="n">
-        <v>5000</v>
-      </c>
+      <c r="I201" s="12" t="n"/>
+      <c r="J201" s="12" t="n"/>
       <c r="K201" s="13">
         <f>E201+F201+G201+H201+I201+J201</f>
         <v/>

</xml_diff>